<commit_message>
Actualitza guia ús Plantilla avaluació
</commit_message>
<xml_diff>
--- a/professorat/avaluació/Plantilla avaluació de Grup de KarmaCli.xlsx
+++ b/professorat/avaluació/Plantilla avaluació de Grup de KarmaCli.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Sofia\Git\_Karma\professorat\avaluació\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1BD5FF3C-D71A-4D02-9C27-8AD277200539}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0593D806-D972-42EE-98F9-6051C96D2517}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="700" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="MÒDUL" sheetId="2" r:id="rId1"/>
@@ -25,6 +25,7 @@
     <sheet name="Alumne1" sheetId="14" r:id="rId10"/>
     <sheet name="Alumne2" sheetId="13" r:id="rId11"/>
     <sheet name="Alumne3" sheetId="12" r:id="rId12"/>
+    <sheet name="Observacions" sheetId="15" r:id="rId13"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -47,11 +48,11 @@
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata">
   <metadataTypes count="1">
     <metadataType name="XLRICHVALUE" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1"/>
   </metadataTypes>
-  <futureMetadata name="XLRICHVALUE" count="5">
+  <futureMetadata name="XLRICHVALUE" count="6">
     <bk>
       <extLst>
         <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
@@ -87,8 +88,15 @@
         </ext>
       </extLst>
     </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="5"/>
+        </ext>
+      </extLst>
+    </bk>
   </futureMetadata>
-  <valueMetadata count="5">
+  <valueMetadata count="6">
     <bk>
       <rc t="1" v="0"/>
     </bk>
@@ -104,12 +112,15 @@
     <bk>
       <rc t="1" v="4"/>
     </bk>
+    <bk>
+      <rc t="1" v="5"/>
+    </bk>
   </valueMetadata>
 </metadata>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="717" uniqueCount="292">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="720" uniqueCount="292">
   <si>
     <t>Nota Mòdul</t>
   </si>
@@ -534,9 +545,6 @@
     <t xml:space="preserve">PDF molt complet, reflexió profunda i ben estructurada. </t>
   </si>
   <si>
-    <t>SPRINT 1</t>
-  </si>
-  <si>
     <t xml:space="preserve">1. Disseny de la interfície i </t>
   </si>
   <si>
@@ -645,9 +653,6 @@
     <t>Vídeo molt ben explicat, amb fluïdesa, claredat, estructura i demostració completa del projecte i el perfil d’usuari.</t>
   </si>
   <si>
-    <t>SPRINT 2</t>
-  </si>
-  <si>
     <t>1.Funcionalitats implementades</t>
   </si>
   <si>
@@ -738,9 +743,6 @@
     <t>Codi net, modular, reutilitzable, ben documentat i amb una estructura clara i coherent.</t>
   </si>
   <si>
-    <t>SPRINT 3</t>
-  </si>
-  <si>
     <t>1. Funcionalitat implementada</t>
   </si>
   <si>
@@ -831,9 +833,6 @@
     <t>Codi net, reutilitzable, ben documentat, modular i fàcil de mantenir.</t>
   </si>
   <si>
-    <t>SPRINT 4</t>
-  </si>
-  <si>
     <t>Inclou gestió de privilegis, consulta de Karma, internacionalització, optimització del rendiment.</t>
   </si>
   <si>
@@ -910,9 +909,6 @@
   </si>
   <si>
     <t>Presentació excel·lent, molt ben explicada, amb fluïdesa, claredat, estructura i demostració completa.</t>
-  </si>
-  <si>
-    <t>SPRINT 5</t>
   </si>
   <si>
     <t>c) S'han identificat els àmbits dutilització de les variables.</t>
@@ -991,6 +987,21 @@
   </si>
   <si>
     <t>Nom Alumne 3</t>
+  </si>
+  <si>
+    <t>EVIDÈNCIA 1 (SPRINT 1)</t>
+  </si>
+  <si>
+    <t>EVIDÈNCIA 2 (SPRINT 2)</t>
+  </si>
+  <si>
+    <t>EVIDÈNCIA 3 (SPRINT 3)</t>
+  </si>
+  <si>
+    <t>EVIDÈNCIA 4 (SPRINT 4)</t>
+  </si>
+  <si>
+    <t>EVIDÈNCIA 5 (SPRINT 5)</t>
   </si>
 </sst>
 </file>
@@ -1676,7 +1687,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="133">
+  <cellXfs count="128">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
@@ -1816,73 +1827,6 @@
     <xf numFmtId="0" fontId="0" fillId="10" borderId="17" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="5" fillId="3" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="5" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="9" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="9" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="9" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="9" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="9" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="9" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="9" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="9" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="11" borderId="24" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1890,24 +1834,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="5" fillId="3" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="5" fillId="3" borderId="32" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="5" fillId="3" borderId="33" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="5" fillId="3" borderId="34" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1915,7 +1841,6 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1928,32 +1853,21 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="32" xfId="0" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="33" xfId="0" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="32" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="33" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="35" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="36" xfId="0" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="37" xfId="0" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="36" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="37" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1969,11 +1883,9 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="34" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -1995,11 +1907,105 @@
     <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="8" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="5" fillId="3" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="5" fillId="3" borderId="32" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="5" fillId="3" borderId="33" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="5" fillId="3" borderId="34" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="5" fillId="3" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="5" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="9" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="9" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="9" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="9" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="9" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="9" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="9" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="9" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="8" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2059,7 +2065,7 @@
 </file>
 
 <file path=xl/richData/rdrichvalue.xml><?xml version="1.0" encoding="utf-8"?>
-<rvData xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="5">
+<rvData xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="6">
   <rv s="0">
     <v>0</v>
     <v>4</v>
@@ -2075,6 +2081,10 @@
   <rv s="0">
     <v>2</v>
     <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>2</v>
+    <v>4</v>
   </rv>
   <rv s="0">
     <v>1</v>
@@ -2422,39 +2432,36 @@
   <cols>
     <col min="1" max="1" width="8.6640625" customWidth="1"/>
     <col min="3" max="3" width="11.88671875" customWidth="1"/>
-    <col min="4" max="4" width="8.88671875" style="118" customWidth="1"/>
-    <col min="5" max="7" width="8.88671875" customWidth="1"/>
+    <col min="4" max="7" width="8.88671875" customWidth="1"/>
     <col min="8" max="8" width="11.44140625" customWidth="1"/>
     <col min="9" max="9" width="13.5546875" customWidth="1"/>
-    <col min="12" max="12" width="8.88671875" style="81"/>
-    <col min="13" max="13" width="5.33203125" style="81" customWidth="1"/>
+    <col min="13" max="13" width="5.33203125" customWidth="1"/>
     <col min="14" max="14" width="11.5546875" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="11.21875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="3:19" ht="6.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="C1" s="93"/>
-      <c r="D1" s="93"/>
-      <c r="E1" s="93"/>
-      <c r="F1" s="93"/>
-      <c r="G1" s="93"/>
+      <c r="C1" s="64"/>
+      <c r="D1" s="64"/>
+      <c r="E1" s="64"/>
+      <c r="F1" s="64"/>
+      <c r="G1" s="64"/>
     </row>
     <row r="2" spans="3:19" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C2" s="122" t="s">
-        <v>273</v>
-      </c>
-      <c r="D2" s="123" t="s">
-        <v>274</v>
-      </c>
-      <c r="E2" s="121"/>
-      <c r="F2" s="121"/>
-      <c r="G2" s="121"/>
-      <c r="H2" s="118"/>
-      <c r="K2" s="85" t="s">
+      <c r="C2" s="85" t="s">
+        <v>268</v>
+      </c>
+      <c r="D2" s="86" t="s">
+        <v>269</v>
+      </c>
+      <c r="E2" s="84"/>
+      <c r="F2" s="84"/>
+      <c r="G2" s="84"/>
+      <c r="K2" s="98" t="s">
         <v>0</v>
       </c>
-      <c r="L2" s="86"/>
-      <c r="M2" s="98"/>
+      <c r="L2" s="99"/>
+      <c r="M2" s="68"/>
       <c r="N2" s="94" t="e" vm="1">
         <f>_xlfn.XLOOKUP(O17/10,R3:R5,S3:S5,,-1)</f>
         <v>#VALUE!</v>
@@ -2471,133 +2478,130 @@
       </c>
     </row>
     <row r="3" spans="3:19" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C3" s="122" t="s">
-        <v>283</v>
-      </c>
-      <c r="D3" s="123" t="s">
-        <v>284</v>
-      </c>
-      <c r="E3" s="121"/>
-      <c r="F3" s="121"/>
-      <c r="G3" s="121"/>
-      <c r="H3" s="118"/>
-      <c r="K3" s="87">
+      <c r="C3" s="85" t="s">
+        <v>278</v>
+      </c>
+      <c r="D3" s="86" t="s">
+        <v>279</v>
+      </c>
+      <c r="E3" s="84"/>
+      <c r="F3" s="84"/>
+      <c r="G3" s="84"/>
+      <c r="K3" s="100">
         <f>O17</f>
         <v>4.9714285714285706</v>
       </c>
-      <c r="L3" s="88"/>
-      <c r="M3" s="98"/>
+      <c r="L3" s="101"/>
+      <c r="M3" s="68"/>
       <c r="N3" s="94"/>
       <c r="O3" s="94"/>
       <c r="Q3" s="21" t="s">
         <v>4</v>
       </c>
-      <c r="R3" s="97">
+      <c r="R3" s="67">
         <v>0</v>
       </c>
-      <c r="S3" s="91" t="e" vm="2">
+      <c r="S3" s="62" t="e" vm="2">
         <v>#VALUE!</v>
       </c>
     </row>
     <row r="4" spans="3:19" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C4" s="122" t="s">
-        <v>269</v>
-      </c>
-      <c r="D4" s="123" t="s">
-        <v>271</v>
-      </c>
-      <c r="E4" s="121"/>
-      <c r="F4" s="121"/>
-      <c r="G4" s="121"/>
-      <c r="H4" s="118"/>
-      <c r="K4" s="87"/>
-      <c r="L4" s="88"/>
-      <c r="M4" s="98"/>
+      <c r="C4" s="85" t="s">
+        <v>264</v>
+      </c>
+      <c r="D4" s="86" t="s">
+        <v>266</v>
+      </c>
+      <c r="E4" s="84"/>
+      <c r="F4" s="84"/>
+      <c r="G4" s="84"/>
+      <c r="K4" s="100"/>
+      <c r="L4" s="101"/>
+      <c r="M4" s="68"/>
       <c r="N4" s="94"/>
       <c r="O4" s="94"/>
       <c r="Q4" s="21" t="s">
         <v>5</v>
       </c>
-      <c r="R4" s="97">
+      <c r="R4" s="67">
         <v>0.45</v>
       </c>
-      <c r="S4" s="91" t="e" vm="3">
+      <c r="S4" s="62" t="e" vm="3">
         <v>#VALUE!</v>
       </c>
     </row>
     <row r="5" spans="3:19" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C5" s="122" t="s">
-        <v>270</v>
-      </c>
-      <c r="D5" s="123" t="s">
-        <v>272</v>
-      </c>
-      <c r="E5" s="121"/>
-      <c r="F5" s="121"/>
-      <c r="G5" s="121"/>
-      <c r="H5" s="118"/>
-      <c r="K5" s="87"/>
-      <c r="L5" s="88"/>
-      <c r="M5" s="98"/>
+      <c r="C5" s="85" t="s">
+        <v>265</v>
+      </c>
+      <c r="D5" s="86" t="s">
+        <v>267</v>
+      </c>
+      <c r="E5" s="84"/>
+      <c r="F5" s="84"/>
+      <c r="G5" s="84"/>
+      <c r="K5" s="100"/>
+      <c r="L5" s="101"/>
+      <c r="M5" s="68"/>
       <c r="N5" s="94"/>
       <c r="O5" s="94"/>
       <c r="Q5" s="21" t="s">
         <v>6</v>
       </c>
-      <c r="R5" s="97">
+      <c r="R5" s="67">
         <v>0.6</v>
       </c>
-      <c r="S5" s="91" t="e" vm="4">
+      <c r="S5" s="62" t="e" vm="4">
         <v>#VALUE!</v>
       </c>
     </row>
     <row r="6" spans="3:19" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="C6" s="92"/>
-      <c r="D6" s="120"/>
-      <c r="K6" s="89"/>
-      <c r="L6" s="90"/>
-      <c r="M6" s="98"/>
+      <c r="C6" s="63"/>
+      <c r="D6" s="61"/>
+      <c r="K6" s="102"/>
+      <c r="L6" s="103"/>
+      <c r="M6" s="68"/>
       <c r="N6" s="94"/>
       <c r="O6" s="94"/>
     </row>
     <row r="7" spans="3:19" ht="24.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C7" s="92"/>
-      <c r="D7" s="120"/>
-      <c r="L7" s="98"/>
-      <c r="M7" s="98"/>
+      <c r="C7" s="63"/>
+      <c r="D7" s="61"/>
+      <c r="L7" s="68"/>
+      <c r="M7" s="68"/>
       <c r="N7" s="94"/>
       <c r="O7" s="94"/>
     </row>
     <row r="8" spans="3:19" x14ac:dyDescent="0.3">
-      <c r="L8" s="98"/>
-      <c r="M8" s="98"/>
+      <c r="L8" s="68"/>
+      <c r="M8" s="68"/>
     </row>
     <row r="9" spans="3:19" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="H9" s="61" t="s">
+      <c r="H9" s="104" t="s">
         <v>8</v>
       </c>
-      <c r="I9" s="61"/>
-      <c r="J9" s="61"/>
-      <c r="K9" s="61"/>
-      <c r="L9" s="61"/>
-      <c r="M9" s="62"/>
-      <c r="N9" s="124" t="s">
+      <c r="I9" s="104"/>
+      <c r="J9" s="104"/>
+      <c r="K9" s="104"/>
+      <c r="L9" s="104"/>
+      <c r="M9" s="105"/>
+      <c r="N9" s="87" t="s">
         <v>7</v>
       </c>
-      <c r="O9" s="125" t="s">
+      <c r="O9" s="88" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="10" spans="3:19" x14ac:dyDescent="0.3">
-      <c r="H10" s="99" t="s">
+      <c r="H10" s="95" t="s">
         <v>10</v>
       </c>
-      <c r="I10" s="100"/>
-      <c r="J10" s="100"/>
-      <c r="K10" s="100"/>
-      <c r="L10" s="100"/>
-      <c r="M10" s="101"/>
-      <c r="N10" s="126">
+      <c r="I10" s="96"/>
+      <c r="J10" s="96"/>
+      <c r="K10" s="96"/>
+      <c r="L10" s="96"/>
+      <c r="M10" s="97"/>
+      <c r="N10" s="89">
         <f>'RA-1'!C8</f>
         <v>0.1</v>
       </c>
@@ -2607,15 +2611,15 @@
       </c>
     </row>
     <row r="11" spans="3:19" x14ac:dyDescent="0.3">
-      <c r="H11" s="99" t="s">
+      <c r="H11" s="95" t="s">
         <v>11</v>
       </c>
-      <c r="I11" s="100"/>
-      <c r="J11" s="100"/>
-      <c r="K11" s="100"/>
-      <c r="L11" s="100"/>
-      <c r="M11" s="101"/>
-      <c r="N11" s="126">
+      <c r="I11" s="96"/>
+      <c r="J11" s="96"/>
+      <c r="K11" s="96"/>
+      <c r="L11" s="96"/>
+      <c r="M11" s="97"/>
+      <c r="N11" s="89">
         <f>'RA-2'!C$8</f>
         <v>0.2</v>
       </c>
@@ -2625,15 +2629,15 @@
       </c>
     </row>
     <row r="12" spans="3:19" x14ac:dyDescent="0.3">
-      <c r="H12" s="99" t="s">
+      <c r="H12" s="95" t="s">
         <v>12</v>
       </c>
-      <c r="I12" s="100"/>
-      <c r="J12" s="100"/>
-      <c r="K12" s="100"/>
-      <c r="L12" s="100"/>
-      <c r="M12" s="101"/>
-      <c r="N12" s="126">
+      <c r="I12" s="96"/>
+      <c r="J12" s="96"/>
+      <c r="K12" s="96"/>
+      <c r="L12" s="96"/>
+      <c r="M12" s="97"/>
+      <c r="N12" s="89">
         <f>'RA-3'!C$8</f>
         <v>0.15</v>
       </c>
@@ -2643,15 +2647,15 @@
       </c>
     </row>
     <row r="13" spans="3:19" x14ac:dyDescent="0.3">
-      <c r="H13" s="99" t="s">
+      <c r="H13" s="95" t="s">
         <v>29</v>
       </c>
-      <c r="I13" s="100"/>
-      <c r="J13" s="100"/>
-      <c r="K13" s="100"/>
-      <c r="L13" s="100"/>
-      <c r="M13" s="101"/>
-      <c r="N13" s="126">
+      <c r="I13" s="96"/>
+      <c r="J13" s="96"/>
+      <c r="K13" s="96"/>
+      <c r="L13" s="96"/>
+      <c r="M13" s="97"/>
+      <c r="N13" s="89">
         <f>'RA-4'!C$8</f>
         <v>0.1</v>
       </c>
@@ -2661,15 +2665,15 @@
       </c>
     </row>
     <row r="14" spans="3:19" x14ac:dyDescent="0.3">
-      <c r="H14" s="99" t="s">
+      <c r="H14" s="95" t="s">
         <v>30</v>
       </c>
-      <c r="I14" s="100"/>
-      <c r="J14" s="100"/>
-      <c r="K14" s="100"/>
-      <c r="L14" s="100"/>
-      <c r="M14" s="101"/>
-      <c r="N14" s="126">
+      <c r="I14" s="96"/>
+      <c r="J14" s="96"/>
+      <c r="K14" s="96"/>
+      <c r="L14" s="96"/>
+      <c r="M14" s="97"/>
+      <c r="N14" s="89">
         <f>'RA-5'!C$8</f>
         <v>0.2</v>
       </c>
@@ -2679,15 +2683,15 @@
       </c>
     </row>
     <row r="15" spans="3:19" x14ac:dyDescent="0.3">
-      <c r="H15" s="99" t="s">
+      <c r="H15" s="95" t="s">
         <v>31</v>
       </c>
-      <c r="I15" s="100"/>
-      <c r="J15" s="100"/>
-      <c r="K15" s="100"/>
-      <c r="L15" s="100"/>
-      <c r="M15" s="101"/>
-      <c r="N15" s="126">
+      <c r="I15" s="96"/>
+      <c r="J15" s="96"/>
+      <c r="K15" s="96"/>
+      <c r="L15" s="96"/>
+      <c r="M15" s="97"/>
+      <c r="N15" s="89">
         <f>'RA-6'!C$8</f>
         <v>0.05</v>
       </c>
@@ -2697,15 +2701,15 @@
       </c>
     </row>
     <row r="16" spans="3:19" x14ac:dyDescent="0.3">
-      <c r="H16" s="99" t="s">
+      <c r="H16" s="95" t="s">
         <v>32</v>
       </c>
-      <c r="I16" s="100"/>
-      <c r="J16" s="100"/>
-      <c r="K16" s="100"/>
-      <c r="L16" s="100"/>
-      <c r="M16" s="101"/>
-      <c r="N16" s="126">
+      <c r="I16" s="96"/>
+      <c r="J16" s="96"/>
+      <c r="K16" s="96"/>
+      <c r="L16" s="96"/>
+      <c r="M16" s="97"/>
+      <c r="N16" s="89">
         <f>'RA-7'!C$8</f>
         <v>0.2</v>
       </c>
@@ -2715,7 +2719,7 @@
       </c>
     </row>
     <row r="17" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="N17" s="127">
+      <c r="N17" s="90">
         <f>SUM(N10:N16)</f>
         <v>1</v>
       </c>
@@ -2724,66 +2728,60 @@
         <v>4.9714285714285706</v>
       </c>
     </row>
-    <row r="19" spans="2:15" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B19" s="81"/>
-    </row>
+    <row r="19" spans="2:15" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="20" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B20" s="28"/>
-      <c r="I20" s="81"/>
-      <c r="J20" s="109"/>
-      <c r="K20" s="110"/>
-      <c r="L20" s="111" t="s">
+      <c r="J20" s="74"/>
+      <c r="K20" s="75"/>
+      <c r="L20" s="76" t="s">
+        <v>272</v>
+      </c>
+      <c r="M20" s="75"/>
+      <c r="N20" s="77"/>
+    </row>
+    <row r="21" spans="2:15" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="J21" s="81">
+        <v>1</v>
+      </c>
+      <c r="K21" s="78">
+        <v>2</v>
+      </c>
+      <c r="L21" s="78">
+        <v>3</v>
+      </c>
+      <c r="M21" s="78">
+        <v>4</v>
+      </c>
+      <c r="N21" s="82">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="22" spans="2:15" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="I22" s="79" t="s">
+        <v>270</v>
+      </c>
+      <c r="J22" s="69" t="s">
+        <v>274</v>
+      </c>
+      <c r="K22" s="70" t="s">
+        <v>273</v>
+      </c>
+      <c r="N22" s="71"/>
+    </row>
+    <row r="23" spans="2:15" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="I23" s="80" t="s">
+        <v>271</v>
+      </c>
+      <c r="J23" s="72"/>
+      <c r="K23" s="32"/>
+      <c r="L23" s="73" t="s">
+        <v>275</v>
+      </c>
+      <c r="M23" s="73" t="s">
+        <v>276</v>
+      </c>
+      <c r="N23" s="83" t="s">
         <v>277</v>
-      </c>
-      <c r="M20" s="110"/>
-      <c r="N20" s="112"/>
-    </row>
-    <row r="21" spans="2:15" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="I21" s="81"/>
-      <c r="J21" s="116">
-        <v>1</v>
-      </c>
-      <c r="K21" s="113">
-        <v>2</v>
-      </c>
-      <c r="L21" s="113">
-        <v>3</v>
-      </c>
-      <c r="M21" s="113">
-        <v>4</v>
-      </c>
-      <c r="N21" s="117">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="22" spans="2:15" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="I22" s="114" t="s">
-        <v>275</v>
-      </c>
-      <c r="J22" s="102" t="s">
-        <v>279</v>
-      </c>
-      <c r="K22" s="103" t="s">
-        <v>278</v>
-      </c>
-      <c r="L22" s="104"/>
-      <c r="M22" s="104"/>
-      <c r="N22" s="105"/>
-    </row>
-    <row r="23" spans="2:15" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="I23" s="115" t="s">
-        <v>276</v>
-      </c>
-      <c r="J23" s="106"/>
-      <c r="K23" s="107"/>
-      <c r="L23" s="108" t="s">
-        <v>280</v>
-      </c>
-      <c r="M23" s="108" t="s">
-        <v>281</v>
-      </c>
-      <c r="N23" s="119" t="s">
-        <v>282</v>
       </c>
     </row>
   </sheetData>
@@ -2810,29 +2808,29 @@
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A1" s="128" t="s">
-        <v>288</v>
-      </c>
-      <c r="B1" s="84" t="s">
-        <v>289</v>
+      <c r="A1" s="91" t="s">
+        <v>283</v>
+      </c>
+      <c r="B1" s="61" t="s">
+        <v>284</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A2" s="129" t="s">
-        <v>286</v>
-      </c>
-      <c r="B2" s="129" t="s">
-        <v>285</v>
-      </c>
-      <c r="C2" s="130" t="s">
-        <v>287</v>
-      </c>
-      <c r="D2" s="130"/>
-      <c r="E2" s="130"/>
-      <c r="F2" s="130"/>
-      <c r="G2" s="130"/>
-      <c r="H2" s="130"/>
-      <c r="I2" s="130"/>
+      <c r="A2" s="92" t="s">
+        <v>281</v>
+      </c>
+      <c r="B2" s="92" t="s">
+        <v>280</v>
+      </c>
+      <c r="C2" s="126" t="s">
+        <v>282</v>
+      </c>
+      <c r="D2" s="126"/>
+      <c r="E2" s="126"/>
+      <c r="F2" s="126"/>
+      <c r="G2" s="126"/>
+      <c r="H2" s="126"/>
+      <c r="I2" s="126"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -2848,29 +2846,29 @@
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A1" s="128" t="s">
-        <v>288</v>
-      </c>
-      <c r="B1" s="84" t="s">
-        <v>290</v>
+      <c r="A1" s="91" t="s">
+        <v>283</v>
+      </c>
+      <c r="B1" s="61" t="s">
+        <v>285</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A2" s="131" t="s">
-        <v>286</v>
-      </c>
-      <c r="B2" s="131" t="s">
-        <v>285</v>
-      </c>
-      <c r="C2" s="132" t="s">
-        <v>287</v>
-      </c>
-      <c r="D2" s="132"/>
-      <c r="E2" s="132"/>
-      <c r="F2" s="132"/>
-      <c r="G2" s="132"/>
-      <c r="H2" s="132"/>
-      <c r="I2" s="132"/>
+      <c r="A2" s="93" t="s">
+        <v>281</v>
+      </c>
+      <c r="B2" s="93" t="s">
+        <v>280</v>
+      </c>
+      <c r="C2" s="127" t="s">
+        <v>282</v>
+      </c>
+      <c r="D2" s="127"/>
+      <c r="E2" s="127"/>
+      <c r="F2" s="127"/>
+      <c r="G2" s="127"/>
+      <c r="H2" s="127"/>
+      <c r="I2" s="127"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -2886,33 +2884,63 @@
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A1" s="128" t="s">
-        <v>288</v>
-      </c>
-      <c r="B1" s="84" t="s">
-        <v>291</v>
+      <c r="A1" s="91" t="s">
+        <v>283</v>
+      </c>
+      <c r="B1" s="61" t="s">
+        <v>286</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A2" s="131" t="s">
-        <v>286</v>
-      </c>
-      <c r="B2" s="131" t="s">
-        <v>285</v>
-      </c>
-      <c r="C2" s="132" t="s">
-        <v>287</v>
-      </c>
-      <c r="D2" s="132"/>
-      <c r="E2" s="132"/>
-      <c r="F2" s="132"/>
-      <c r="G2" s="132"/>
-      <c r="H2" s="132"/>
-      <c r="I2" s="132"/>
+      <c r="A2" s="93" t="s">
+        <v>281</v>
+      </c>
+      <c r="B2" s="93" t="s">
+        <v>280</v>
+      </c>
+      <c r="C2" s="127" t="s">
+        <v>282</v>
+      </c>
+      <c r="D2" s="127"/>
+      <c r="E2" s="127"/>
+      <c r="F2" s="127"/>
+      <c r="G2" s="127"/>
+      <c r="H2" s="127"/>
+      <c r="I2" s="127"/>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="C2:I2"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{42DB9054-9A45-4344-B058-45A4C531AA5E}">
+  <dimension ref="A1:I1"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A1" s="92" t="s">
+        <v>281</v>
+      </c>
+      <c r="B1" s="92" t="s">
+        <v>280</v>
+      </c>
+      <c r="C1" s="126" t="s">
+        <v>282</v>
+      </c>
+      <c r="D1" s="126"/>
+      <c r="E1" s="126"/>
+      <c r="F1" s="126"/>
+      <c r="G1" s="126"/>
+      <c r="H1" s="126"/>
+      <c r="I1" s="126"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="C1:I1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -2934,31 +2962,31 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="61.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="64" t="s">
+      <c r="A1" s="106" t="s">
         <v>38</v>
       </c>
-      <c r="B1" s="64"/>
-      <c r="C1" s="64"/>
-      <c r="D1" s="64"/>
-      <c r="E1" s="64"/>
-      <c r="F1" s="64"/>
-      <c r="G1" s="64"/>
-      <c r="H1" s="64"/>
-      <c r="I1" s="64"/>
-      <c r="J1" s="64"/>
-      <c r="K1" s="64"/>
-      <c r="L1" s="64"/>
+      <c r="B1" s="106"/>
+      <c r="C1" s="106"/>
+      <c r="D1" s="106"/>
+      <c r="E1" s="106"/>
+      <c r="F1" s="106"/>
+      <c r="G1" s="106"/>
+      <c r="H1" s="106"/>
+      <c r="I1" s="106"/>
+      <c r="J1" s="106"/>
+      <c r="K1" s="106"/>
+      <c r="L1" s="106"/>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="C3" s="65">
+      <c r="C3" s="107">
         <f>D3*C8</f>
         <v>0.7200000000000002</v>
       </c>
-      <c r="D3" s="66">
+      <c r="D3" s="108">
         <f>I17*10</f>
         <v>7.2000000000000011</v>
       </c>
-      <c r="E3" s="67"/>
+      <c r="E3" s="109"/>
       <c r="F3" s="11" t="s">
         <v>1</v>
       </c>
@@ -2985,16 +3013,16 @@
       </c>
     </row>
     <row r="4" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C4" s="65"/>
-      <c r="D4" s="66"/>
-      <c r="E4" s="67"/>
+      <c r="C4" s="107"/>
+      <c r="D4" s="108"/>
+      <c r="E4" s="109"/>
       <c r="F4" s="12" t="s">
         <v>4</v>
       </c>
-      <c r="G4" s="5">
+      <c r="G4" s="67">
         <v>0</v>
       </c>
-      <c r="H4" s="95" t="e" vm="2">
+      <c r="H4" s="65" t="e" vm="2">
         <v>#VALUE!</v>
       </c>
       <c r="J4" s="10" t="s">
@@ -3014,16 +3042,16 @@
       </c>
     </row>
     <row r="5" spans="1:15" ht="21" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C5" s="65"/>
-      <c r="D5" s="66"/>
-      <c r="E5" s="67"/>
+      <c r="C5" s="107"/>
+      <c r="D5" s="108"/>
+      <c r="E5" s="109"/>
       <c r="F5" s="13" t="s">
         <v>5</v>
       </c>
-      <c r="G5" s="2">
-        <v>0.6</v>
-      </c>
-      <c r="H5" s="96" t="e" vm="3">
+      <c r="G5" s="67">
+        <v>0.45</v>
+      </c>
+      <c r="H5" s="66" t="e" vm="3">
         <v>#VALUE!</v>
       </c>
       <c r="J5" s="10" t="s">
@@ -3043,16 +3071,16 @@
       </c>
     </row>
     <row r="6" spans="1:15" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C6" s="65"/>
-      <c r="D6" s="66"/>
-      <c r="E6" s="67"/>
+      <c r="C6" s="107"/>
+      <c r="D6" s="108"/>
+      <c r="E6" s="109"/>
       <c r="F6" s="13" t="s">
         <v>6</v>
       </c>
-      <c r="G6" s="2">
-        <v>0.9</v>
-      </c>
-      <c r="H6" s="96" t="e" vm="4">
+      <c r="G6" s="67">
+        <v>0.6</v>
+      </c>
+      <c r="H6" s="66" t="e" vm="4">
         <v>#VALUE!</v>
       </c>
       <c r="J6" s="10" t="s">
@@ -3072,12 +3100,12 @@
       </c>
     </row>
     <row r="7" spans="1:15" ht="24.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="F7" s="59" t="e" vm="1">
+      <c r="F7" s="110" t="e" vm="5">
         <f>_xlfn.XLOOKUP(H17,G4:G6,H4:H6,,-1)</f>
         <v>#VALUE!</v>
       </c>
-      <c r="G7" s="59"/>
-      <c r="H7" s="59"/>
+      <c r="G7" s="110"/>
+      <c r="H7" s="110"/>
       <c r="J7" s="10" t="s">
         <v>40</v>
       </c>
@@ -3101,9 +3129,9 @@
       <c r="C8" s="15">
         <v>0.1</v>
       </c>
-      <c r="F8" s="59"/>
-      <c r="G8" s="59"/>
-      <c r="H8" s="59"/>
+      <c r="F8" s="110"/>
+      <c r="G8" s="110"/>
+      <c r="H8" s="110"/>
       <c r="J8" s="7" t="s">
         <v>14</v>
       </c>
@@ -3121,14 +3149,14 @@
       </c>
     </row>
     <row r="9" spans="1:15" ht="70.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C9" s="60" t="s">
+      <c r="C9" s="111" t="s">
         <v>27</v>
       </c>
-      <c r="D9" s="60"/>
-      <c r="E9" s="60"/>
-      <c r="F9" s="59"/>
-      <c r="G9" s="59"/>
-      <c r="H9" s="59"/>
+      <c r="D9" s="111"/>
+      <c r="E9" s="111"/>
+      <c r="F9" s="110"/>
+      <c r="G9" s="110"/>
+      <c r="H9" s="110"/>
       <c r="J9" s="19" t="s">
         <v>39</v>
       </c>
@@ -3146,14 +3174,14 @@
       </c>
     </row>
     <row r="10" spans="1:15" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="61" t="s">
+      <c r="A10" s="104" t="s">
         <v>15</v>
       </c>
-      <c r="B10" s="61"/>
-      <c r="C10" s="61"/>
-      <c r="D10" s="61"/>
-      <c r="E10" s="61"/>
-      <c r="F10" s="62"/>
+      <c r="B10" s="104"/>
+      <c r="C10" s="104"/>
+      <c r="D10" s="104"/>
+      <c r="E10" s="104"/>
+      <c r="F10" s="105"/>
       <c r="G10" s="6" t="s">
         <v>7</v>
       </c>
@@ -3183,14 +3211,14 @@
       </c>
     </row>
     <row r="11" spans="1:15" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="63" t="s">
+      <c r="A11" s="112" t="s">
         <v>46</v>
       </c>
-      <c r="B11" s="63"/>
-      <c r="C11" s="63"/>
-      <c r="D11" s="63"/>
-      <c r="E11" s="63"/>
-      <c r="F11" s="63"/>
+      <c r="B11" s="112"/>
+      <c r="C11" s="112"/>
+      <c r="D11" s="112"/>
+      <c r="E11" s="112"/>
+      <c r="F11" s="112"/>
       <c r="G11" s="22">
         <v>0.15</v>
       </c>
@@ -3212,23 +3240,23 @@
       <c r="N11" s="31"/>
     </row>
     <row r="12" spans="1:15" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="63" t="s">
+      <c r="A12" s="112" t="s">
         <v>47</v>
       </c>
-      <c r="B12" s="63"/>
-      <c r="C12" s="63"/>
-      <c r="D12" s="63"/>
-      <c r="E12" s="63"/>
-      <c r="F12" s="63"/>
+      <c r="B12" s="112"/>
+      <c r="C12" s="112"/>
+      <c r="D12" s="112"/>
+      <c r="E12" s="112"/>
+      <c r="F12" s="112"/>
       <c r="G12" s="22">
         <v>0.2</v>
       </c>
       <c r="H12" s="22">
-        <f t="shared" ref="H11:H16" si="0">I12*G12</f>
+        <f t="shared" ref="H12:H16" si="0">I12*G12</f>
         <v>0.14400000000000002</v>
       </c>
       <c r="I12" s="22">
-        <f t="shared" ref="I11:I16" si="1">IFERROR(IF(SUM(J12:N12)/COUNT(J12:N12)&gt;=10,1,(SUM(J12:N12)/COUNT(J12:N12)/10)),0)</f>
+        <f t="shared" ref="I12:I16" si="1">IFERROR(IF(SUM(J12:N12)/COUNT(J12:N12)&gt;=10,1,(SUM(J12:N12)/COUNT(J12:N12)/10)),0)</f>
         <v>0.72000000000000008</v>
       </c>
       <c r="J12" s="30">
@@ -3241,14 +3269,14 @@
       <c r="N12" s="31"/>
     </row>
     <row r="13" spans="1:15" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="63" t="s">
+      <c r="A13" s="112" t="s">
         <v>48</v>
       </c>
-      <c r="B13" s="63"/>
-      <c r="C13" s="63"/>
-      <c r="D13" s="63"/>
-      <c r="E13" s="63"/>
-      <c r="F13" s="63"/>
+      <c r="B13" s="112"/>
+      <c r="C13" s="112"/>
+      <c r="D13" s="112"/>
+      <c r="E13" s="112"/>
+      <c r="F13" s="112"/>
       <c r="G13" s="22">
         <v>0.15</v>
       </c>
@@ -3270,14 +3298,14 @@
       <c r="N13" s="31"/>
     </row>
     <row r="14" spans="1:15" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="63" t="s">
+      <c r="A14" s="112" t="s">
         <v>49</v>
       </c>
-      <c r="B14" s="63"/>
-      <c r="C14" s="63"/>
-      <c r="D14" s="63"/>
-      <c r="E14" s="63"/>
-      <c r="F14" s="63"/>
+      <c r="B14" s="112"/>
+      <c r="C14" s="112"/>
+      <c r="D14" s="112"/>
+      <c r="E14" s="112"/>
+      <c r="F14" s="112"/>
       <c r="G14" s="22">
         <v>0.15</v>
       </c>
@@ -3299,14 +3327,14 @@
       <c r="N14" s="31"/>
     </row>
     <row r="15" spans="1:15" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="63" t="s">
+      <c r="A15" s="112" t="s">
         <v>50</v>
       </c>
-      <c r="B15" s="63"/>
-      <c r="C15" s="63"/>
-      <c r="D15" s="63"/>
-      <c r="E15" s="63"/>
-      <c r="F15" s="63"/>
+      <c r="B15" s="112"/>
+      <c r="C15" s="112"/>
+      <c r="D15" s="112"/>
+      <c r="E15" s="112"/>
+      <c r="F15" s="112"/>
       <c r="G15" s="22">
         <v>0.15</v>
       </c>
@@ -3328,14 +3356,14 @@
       <c r="N15" s="31"/>
     </row>
     <row r="16" spans="1:15" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="63" t="s">
+      <c r="A16" s="112" t="s">
         <v>51</v>
       </c>
-      <c r="B16" s="63"/>
-      <c r="C16" s="63"/>
-      <c r="D16" s="63"/>
-      <c r="E16" s="63"/>
-      <c r="F16" s="63"/>
+      <c r="B16" s="112"/>
+      <c r="C16" s="112"/>
+      <c r="D16" s="112"/>
+      <c r="E16" s="112"/>
+      <c r="F16" s="112"/>
       <c r="G16" s="22">
         <v>0.2</v>
       </c>
@@ -3390,11 +3418,6 @@
     </row>
   </sheetData>
   <mergeCells count="12">
-    <mergeCell ref="A1:L1"/>
-    <mergeCell ref="C3:C6"/>
-    <mergeCell ref="D3:E6"/>
-    <mergeCell ref="F7:H9"/>
-    <mergeCell ref="C9:E9"/>
     <mergeCell ref="A13:F13"/>
     <mergeCell ref="A14:F14"/>
     <mergeCell ref="A15:F15"/>
@@ -3402,6 +3425,11 @@
     <mergeCell ref="A10:F10"/>
     <mergeCell ref="A12:F12"/>
     <mergeCell ref="A11:F11"/>
+    <mergeCell ref="A1:L1"/>
+    <mergeCell ref="C3:C6"/>
+    <mergeCell ref="D3:E6"/>
+    <mergeCell ref="F7:H9"/>
+    <mergeCell ref="C9:E9"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -3423,32 +3451,32 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="61.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="64" t="s">
+      <c r="A1" s="106" t="s">
         <v>52</v>
       </c>
-      <c r="B1" s="64"/>
-      <c r="C1" s="64"/>
-      <c r="D1" s="64"/>
-      <c r="E1" s="64"/>
-      <c r="F1" s="64"/>
-      <c r="G1" s="64"/>
-      <c r="H1" s="64"/>
-      <c r="I1" s="64"/>
-      <c r="J1" s="64"/>
-      <c r="K1" s="64"/>
-      <c r="L1" s="64"/>
-      <c r="M1" s="64"/>
+      <c r="B1" s="106"/>
+      <c r="C1" s="106"/>
+      <c r="D1" s="106"/>
+      <c r="E1" s="106"/>
+      <c r="F1" s="106"/>
+      <c r="G1" s="106"/>
+      <c r="H1" s="106"/>
+      <c r="I1" s="106"/>
+      <c r="J1" s="106"/>
+      <c r="K1" s="106"/>
+      <c r="L1" s="106"/>
+      <c r="M1" s="106"/>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="C3" s="65">
+      <c r="C3" s="107">
         <f>D3*C8</f>
         <v>1.44</v>
       </c>
-      <c r="D3" s="66">
+      <c r="D3" s="108">
         <f>I19*10</f>
         <v>7.1999999999999993</v>
       </c>
-      <c r="E3" s="67"/>
+      <c r="E3" s="109"/>
       <c r="F3" s="11" t="s">
         <v>1</v>
       </c>
@@ -3475,9 +3503,9 @@
       </c>
     </row>
     <row r="4" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C4" s="65"/>
-      <c r="D4" s="66"/>
-      <c r="E4" s="67"/>
+      <c r="C4" s="107"/>
+      <c r="D4" s="108"/>
+      <c r="E4" s="109"/>
       <c r="F4" s="12" t="s">
         <v>4</v>
       </c>
@@ -3504,9 +3532,9 @@
       </c>
     </row>
     <row r="5" spans="1:15" ht="21" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C5" s="65"/>
-      <c r="D5" s="66"/>
-      <c r="E5" s="67"/>
+      <c r="C5" s="107"/>
+      <c r="D5" s="108"/>
+      <c r="E5" s="109"/>
       <c r="F5" s="13" t="s">
         <v>5</v>
       </c>
@@ -3533,9 +3561,9 @@
       </c>
     </row>
     <row r="6" spans="1:15" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C6" s="65"/>
-      <c r="D6" s="66"/>
-      <c r="E6" s="67"/>
+      <c r="C6" s="107"/>
+      <c r="D6" s="108"/>
+      <c r="E6" s="109"/>
       <c r="F6" s="13" t="s">
         <v>6</v>
       </c>
@@ -3562,12 +3590,12 @@
       </c>
     </row>
     <row r="7" spans="1:15" ht="24.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="F7" s="59" t="e" vm="1">
+      <c r="F7" s="110" t="e" vm="1">
         <f>_xlfn.XLOOKUP(H19,G4:G6,H4:H6,,-1)</f>
         <v>#VALUE!</v>
       </c>
-      <c r="G7" s="59"/>
-      <c r="H7" s="59"/>
+      <c r="G7" s="110"/>
+      <c r="H7" s="110"/>
       <c r="J7" s="10" t="s">
         <v>40</v>
       </c>
@@ -3591,9 +3619,9 @@
       <c r="C8" s="15">
         <v>0.2</v>
       </c>
-      <c r="F8" s="59"/>
-      <c r="G8" s="59"/>
-      <c r="H8" s="59"/>
+      <c r="F8" s="110"/>
+      <c r="G8" s="110"/>
+      <c r="H8" s="110"/>
       <c r="J8" s="7" t="s">
         <v>14</v>
       </c>
@@ -3611,14 +3639,14 @@
       </c>
     </row>
     <row r="9" spans="1:15" ht="70.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C9" s="60" t="s">
+      <c r="C9" s="111" t="s">
         <v>25</v>
       </c>
-      <c r="D9" s="60"/>
-      <c r="E9" s="60"/>
-      <c r="F9" s="59"/>
-      <c r="G9" s="59"/>
-      <c r="H9" s="59"/>
+      <c r="D9" s="111"/>
+      <c r="E9" s="111"/>
+      <c r="F9" s="110"/>
+      <c r="G9" s="110"/>
+      <c r="H9" s="110"/>
       <c r="J9" s="19" t="s">
         <v>39</v>
       </c>
@@ -3636,14 +3664,14 @@
       </c>
     </row>
     <row r="10" spans="1:15" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="68" t="s">
+      <c r="A10" s="113" t="s">
         <v>15</v>
       </c>
-      <c r="B10" s="68"/>
-      <c r="C10" s="68"/>
-      <c r="D10" s="68"/>
-      <c r="E10" s="68"/>
-      <c r="F10" s="69"/>
+      <c r="B10" s="113"/>
+      <c r="C10" s="113"/>
+      <c r="D10" s="113"/>
+      <c r="E10" s="113"/>
+      <c r="F10" s="114"/>
       <c r="G10" s="6" t="s">
         <v>7</v>
       </c>
@@ -3673,14 +3701,14 @@
       </c>
     </row>
     <row r="11" spans="1:15" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="63" t="s">
+      <c r="A11" s="112" t="s">
         <v>58</v>
       </c>
-      <c r="B11" s="63"/>
-      <c r="C11" s="63"/>
-      <c r="D11" s="63"/>
-      <c r="E11" s="63"/>
-      <c r="F11" s="63"/>
+      <c r="B11" s="112"/>
+      <c r="C11" s="112"/>
+      <c r="D11" s="112"/>
+      <c r="E11" s="112"/>
+      <c r="F11" s="112"/>
       <c r="G11" s="22">
         <v>0.05</v>
       </c>
@@ -3702,14 +3730,14 @@
       <c r="N11" s="31"/>
     </row>
     <row r="12" spans="1:15" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="63" t="s">
+      <c r="A12" s="112" t="s">
         <v>59</v>
       </c>
-      <c r="B12" s="63"/>
-      <c r="C12" s="63"/>
-      <c r="D12" s="63"/>
-      <c r="E12" s="63"/>
-      <c r="F12" s="63"/>
+      <c r="B12" s="112"/>
+      <c r="C12" s="112"/>
+      <c r="D12" s="112"/>
+      <c r="E12" s="112"/>
+      <c r="F12" s="112"/>
       <c r="G12" s="22">
         <v>0.15</v>
       </c>
@@ -3731,14 +3759,14 @@
       <c r="N12" s="31"/>
     </row>
     <row r="13" spans="1:15" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="63" t="s">
-        <v>268</v>
-      </c>
-      <c r="B13" s="63"/>
-      <c r="C13" s="63"/>
-      <c r="D13" s="63"/>
-      <c r="E13" s="63"/>
-      <c r="F13" s="63"/>
+      <c r="A13" s="112" t="s">
+        <v>263</v>
+      </c>
+      <c r="B13" s="112"/>
+      <c r="C13" s="112"/>
+      <c r="D13" s="112"/>
+      <c r="E13" s="112"/>
+      <c r="F13" s="112"/>
       <c r="G13" s="22">
         <v>0.15</v>
       </c>
@@ -3760,14 +3788,14 @@
       <c r="N13" s="31"/>
     </row>
     <row r="14" spans="1:15" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="63" t="s">
+      <c r="A14" s="112" t="s">
         <v>60</v>
       </c>
-      <c r="B14" s="63"/>
-      <c r="C14" s="63"/>
-      <c r="D14" s="63"/>
-      <c r="E14" s="63"/>
-      <c r="F14" s="63"/>
+      <c r="B14" s="112"/>
+      <c r="C14" s="112"/>
+      <c r="D14" s="112"/>
+      <c r="E14" s="112"/>
+      <c r="F14" s="112"/>
       <c r="G14" s="22">
         <v>0.15</v>
       </c>
@@ -3789,14 +3817,14 @@
       <c r="N14" s="31"/>
     </row>
     <row r="15" spans="1:15" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="63" t="s">
+      <c r="A15" s="112" t="s">
         <v>61</v>
       </c>
-      <c r="B15" s="63"/>
-      <c r="C15" s="63"/>
-      <c r="D15" s="63"/>
-      <c r="E15" s="63"/>
-      <c r="F15" s="63"/>
+      <c r="B15" s="112"/>
+      <c r="C15" s="112"/>
+      <c r="D15" s="112"/>
+      <c r="E15" s="112"/>
+      <c r="F15" s="112"/>
       <c r="G15" s="22">
         <v>0.15</v>
       </c>
@@ -3818,14 +3846,14 @@
       <c r="N15" s="31"/>
     </row>
     <row r="16" spans="1:15" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="63" t="s">
+      <c r="A16" s="112" t="s">
         <v>62</v>
       </c>
-      <c r="B16" s="63"/>
-      <c r="C16" s="63"/>
-      <c r="D16" s="63"/>
-      <c r="E16" s="63"/>
-      <c r="F16" s="63"/>
+      <c r="B16" s="112"/>
+      <c r="C16" s="112"/>
+      <c r="D16" s="112"/>
+      <c r="E16" s="112"/>
+      <c r="F16" s="112"/>
       <c r="G16" s="22">
         <v>0.1</v>
       </c>
@@ -3847,14 +3875,14 @@
       <c r="N16" s="31"/>
     </row>
     <row r="17" spans="1:14" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="63" t="s">
+      <c r="A17" s="112" t="s">
         <v>63</v>
       </c>
-      <c r="B17" s="63"/>
-      <c r="C17" s="63"/>
-      <c r="D17" s="63"/>
-      <c r="E17" s="63"/>
-      <c r="F17" s="63"/>
+      <c r="B17" s="112"/>
+      <c r="C17" s="112"/>
+      <c r="D17" s="112"/>
+      <c r="E17" s="112"/>
+      <c r="F17" s="112"/>
       <c r="G17" s="22">
         <v>0.1</v>
       </c>
@@ -3876,14 +3904,14 @@
       <c r="N17" s="31"/>
     </row>
     <row r="18" spans="1:14" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="63" t="s">
+      <c r="A18" s="112" t="s">
         <v>64</v>
       </c>
-      <c r="B18" s="63"/>
-      <c r="C18" s="63"/>
-      <c r="D18" s="63"/>
-      <c r="E18" s="63"/>
-      <c r="F18" s="63"/>
+      <c r="B18" s="112"/>
+      <c r="C18" s="112"/>
+      <c r="D18" s="112"/>
+      <c r="E18" s="112"/>
+      <c r="F18" s="112"/>
       <c r="G18" s="22">
         <v>0.15</v>
       </c>
@@ -3938,6 +3966,12 @@
     </row>
   </sheetData>
   <mergeCells count="14">
+    <mergeCell ref="A18:F18"/>
+    <mergeCell ref="F7:H9"/>
+    <mergeCell ref="C9:E9"/>
+    <mergeCell ref="A10:F10"/>
+    <mergeCell ref="A11:F11"/>
+    <mergeCell ref="A12:F12"/>
     <mergeCell ref="A1:M1"/>
     <mergeCell ref="A17:F17"/>
     <mergeCell ref="A14:F14"/>
@@ -3946,12 +3980,6 @@
     <mergeCell ref="D3:E6"/>
     <mergeCell ref="C3:C6"/>
     <mergeCell ref="A13:F13"/>
-    <mergeCell ref="A18:F18"/>
-    <mergeCell ref="F7:H9"/>
-    <mergeCell ref="C9:E9"/>
-    <mergeCell ref="A10:F10"/>
-    <mergeCell ref="A11:F11"/>
-    <mergeCell ref="A12:F12"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -3973,32 +4001,32 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="61.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="64" t="s">
+      <c r="A1" s="106" t="s">
         <v>53</v>
       </c>
-      <c r="B1" s="64"/>
-      <c r="C1" s="64"/>
-      <c r="D1" s="64"/>
-      <c r="E1" s="64"/>
-      <c r="F1" s="64"/>
-      <c r="G1" s="64"/>
-      <c r="H1" s="64"/>
-      <c r="I1" s="64"/>
-      <c r="J1" s="64"/>
-      <c r="K1" s="64"/>
-      <c r="L1" s="64"/>
-      <c r="M1" s="64"/>
+      <c r="B1" s="106"/>
+      <c r="C1" s="106"/>
+      <c r="D1" s="106"/>
+      <c r="E1" s="106"/>
+      <c r="F1" s="106"/>
+      <c r="G1" s="106"/>
+      <c r="H1" s="106"/>
+      <c r="I1" s="106"/>
+      <c r="J1" s="106"/>
+      <c r="K1" s="106"/>
+      <c r="L1" s="106"/>
+      <c r="M1" s="106"/>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="C3" s="65">
+      <c r="C3" s="107">
         <f>D3*C8</f>
         <v>1.0199999999999998</v>
       </c>
-      <c r="D3" s="66">
+      <c r="D3" s="108">
         <f>I19*10</f>
         <v>6.7999999999999989</v>
       </c>
-      <c r="E3" s="67"/>
+      <c r="E3" s="109"/>
       <c r="F3" s="11" t="s">
         <v>1</v>
       </c>
@@ -4025,9 +4053,9 @@
       </c>
     </row>
     <row r="4" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C4" s="65"/>
-      <c r="D4" s="66"/>
-      <c r="E4" s="67"/>
+      <c r="C4" s="107"/>
+      <c r="D4" s="108"/>
+      <c r="E4" s="109"/>
       <c r="F4" s="12" t="s">
         <v>4</v>
       </c>
@@ -4054,9 +4082,9 @@
       </c>
     </row>
     <row r="5" spans="1:15" ht="21" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C5" s="65"/>
-      <c r="D5" s="66"/>
-      <c r="E5" s="67"/>
+      <c r="C5" s="107"/>
+      <c r="D5" s="108"/>
+      <c r="E5" s="109"/>
       <c r="F5" s="13" t="s">
         <v>5</v>
       </c>
@@ -4083,9 +4111,9 @@
       </c>
     </row>
     <row r="6" spans="1:15" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C6" s="65"/>
-      <c r="D6" s="66"/>
-      <c r="E6" s="67"/>
+      <c r="C6" s="107"/>
+      <c r="D6" s="108"/>
+      <c r="E6" s="109"/>
       <c r="F6" s="13" t="s">
         <v>6</v>
       </c>
@@ -4112,12 +4140,12 @@
       </c>
     </row>
     <row r="7" spans="1:15" ht="24.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="F7" s="59" t="e" vm="1">
+      <c r="F7" s="110" t="e" vm="1">
         <f>_xlfn.XLOOKUP(H19,G4:G6,H4:H6,,-1)</f>
         <v>#VALUE!</v>
       </c>
-      <c r="G7" s="59"/>
-      <c r="H7" s="59"/>
+      <c r="G7" s="110"/>
+      <c r="H7" s="110"/>
       <c r="J7" s="10" t="s">
         <v>40</v>
       </c>
@@ -4141,9 +4169,9 @@
       <c r="C8" s="15">
         <v>0.15</v>
       </c>
-      <c r="F8" s="59"/>
-      <c r="G8" s="59"/>
-      <c r="H8" s="59"/>
+      <c r="F8" s="110"/>
+      <c r="G8" s="110"/>
+      <c r="H8" s="110"/>
       <c r="J8" s="7" t="s">
         <v>14</v>
       </c>
@@ -4161,14 +4189,14 @@
       </c>
     </row>
     <row r="9" spans="1:15" ht="70.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C9" s="60" t="s">
+      <c r="C9" s="111" t="s">
         <v>33</v>
       </c>
-      <c r="D9" s="60"/>
-      <c r="E9" s="60"/>
-      <c r="F9" s="59"/>
-      <c r="G9" s="59"/>
-      <c r="H9" s="59"/>
+      <c r="D9" s="111"/>
+      <c r="E9" s="111"/>
+      <c r="F9" s="110"/>
+      <c r="G9" s="110"/>
+      <c r="H9" s="110"/>
       <c r="J9" s="19" t="s">
         <v>39</v>
       </c>
@@ -4186,14 +4214,14 @@
       </c>
     </row>
     <row r="10" spans="1:15" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="68" t="s">
+      <c r="A10" s="113" t="s">
         <v>15</v>
       </c>
-      <c r="B10" s="68"/>
-      <c r="C10" s="68"/>
-      <c r="D10" s="68"/>
-      <c r="E10" s="68"/>
-      <c r="F10" s="69"/>
+      <c r="B10" s="113"/>
+      <c r="C10" s="113"/>
+      <c r="D10" s="113"/>
+      <c r="E10" s="113"/>
+      <c r="F10" s="114"/>
       <c r="G10" s="6" t="s">
         <v>7</v>
       </c>
@@ -4223,14 +4251,14 @@
       </c>
     </row>
     <row r="11" spans="1:15" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="63" t="s">
+      <c r="A11" s="112" t="s">
         <v>65</v>
       </c>
-      <c r="B11" s="63"/>
-      <c r="C11" s="63"/>
-      <c r="D11" s="63"/>
-      <c r="E11" s="63"/>
-      <c r="F11" s="63"/>
+      <c r="B11" s="112"/>
+      <c r="C11" s="112"/>
+      <c r="D11" s="112"/>
+      <c r="E11" s="112"/>
+      <c r="F11" s="112"/>
       <c r="G11" s="27">
         <v>0.15</v>
       </c>
@@ -4255,14 +4283,14 @@
       </c>
     </row>
     <row r="12" spans="1:15" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="63" t="s">
+      <c r="A12" s="112" t="s">
         <v>66</v>
       </c>
-      <c r="B12" s="63"/>
-      <c r="C12" s="63"/>
-      <c r="D12" s="63"/>
-      <c r="E12" s="63"/>
-      <c r="F12" s="63"/>
+      <c r="B12" s="112"/>
+      <c r="C12" s="112"/>
+      <c r="D12" s="112"/>
+      <c r="E12" s="112"/>
+      <c r="F12" s="112"/>
       <c r="G12" s="27">
         <v>0.15</v>
       </c>
@@ -4287,14 +4315,14 @@
       </c>
     </row>
     <row r="13" spans="1:15" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="63" t="s">
+      <c r="A13" s="112" t="s">
         <v>67</v>
       </c>
-      <c r="B13" s="63"/>
-      <c r="C13" s="63"/>
-      <c r="D13" s="63"/>
-      <c r="E13" s="63"/>
-      <c r="F13" s="63"/>
+      <c r="B13" s="112"/>
+      <c r="C13" s="112"/>
+      <c r="D13" s="112"/>
+      <c r="E13" s="112"/>
+      <c r="F13" s="112"/>
       <c r="G13" s="27">
         <v>0.1</v>
       </c>
@@ -4319,14 +4347,14 @@
       </c>
     </row>
     <row r="14" spans="1:15" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="63" t="s">
+      <c r="A14" s="112" t="s">
         <v>68</v>
       </c>
-      <c r="B14" s="63"/>
-      <c r="C14" s="63"/>
-      <c r="D14" s="63"/>
-      <c r="E14" s="63"/>
-      <c r="F14" s="63"/>
+      <c r="B14" s="112"/>
+      <c r="C14" s="112"/>
+      <c r="D14" s="112"/>
+      <c r="E14" s="112"/>
+      <c r="F14" s="112"/>
       <c r="G14" s="27">
         <v>0.1</v>
       </c>
@@ -4351,14 +4379,14 @@
       </c>
     </row>
     <row r="15" spans="1:15" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="63" t="s">
+      <c r="A15" s="112" t="s">
         <v>69</v>
       </c>
-      <c r="B15" s="63"/>
-      <c r="C15" s="63"/>
-      <c r="D15" s="63"/>
-      <c r="E15" s="63"/>
-      <c r="F15" s="63"/>
+      <c r="B15" s="112"/>
+      <c r="C15" s="112"/>
+      <c r="D15" s="112"/>
+      <c r="E15" s="112"/>
+      <c r="F15" s="112"/>
       <c r="G15" s="27">
         <v>0.125</v>
       </c>
@@ -4383,14 +4411,14 @@
       </c>
     </row>
     <row r="16" spans="1:15" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="63" t="s">
+      <c r="A16" s="112" t="s">
         <v>70</v>
       </c>
-      <c r="B16" s="63"/>
-      <c r="C16" s="63"/>
-      <c r="D16" s="63"/>
-      <c r="E16" s="63"/>
-      <c r="F16" s="63"/>
+      <c r="B16" s="112"/>
+      <c r="C16" s="112"/>
+      <c r="D16" s="112"/>
+      <c r="E16" s="112"/>
+      <c r="F16" s="112"/>
       <c r="G16" s="27">
         <v>0.125</v>
       </c>
@@ -4415,14 +4443,14 @@
       </c>
     </row>
     <row r="17" spans="1:14" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="63" t="s">
+      <c r="A17" s="112" t="s">
         <v>71</v>
       </c>
-      <c r="B17" s="63"/>
-      <c r="C17" s="63"/>
-      <c r="D17" s="63"/>
-      <c r="E17" s="63"/>
-      <c r="F17" s="63"/>
+      <c r="B17" s="112"/>
+      <c r="C17" s="112"/>
+      <c r="D17" s="112"/>
+      <c r="E17" s="112"/>
+      <c r="F17" s="112"/>
       <c r="G17" s="27">
         <v>0.125</v>
       </c>
@@ -4447,14 +4475,14 @@
       </c>
     </row>
     <row r="18" spans="1:14" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="63" t="s">
+      <c r="A18" s="112" t="s">
         <v>72</v>
       </c>
-      <c r="B18" s="63"/>
-      <c r="C18" s="63"/>
-      <c r="D18" s="63"/>
-      <c r="E18" s="63"/>
-      <c r="F18" s="63"/>
+      <c r="B18" s="112"/>
+      <c r="C18" s="112"/>
+      <c r="D18" s="112"/>
+      <c r="E18" s="112"/>
+      <c r="F18" s="112"/>
       <c r="G18" s="27">
         <v>0.125</v>
       </c>
@@ -4512,6 +4540,13 @@
     </row>
   </sheetData>
   <mergeCells count="14">
+    <mergeCell ref="A18:F18"/>
+    <mergeCell ref="C3:C6"/>
+    <mergeCell ref="D3:E6"/>
+    <mergeCell ref="F7:H9"/>
+    <mergeCell ref="C9:E9"/>
+    <mergeCell ref="A10:F10"/>
+    <mergeCell ref="A11:F11"/>
     <mergeCell ref="A1:M1"/>
     <mergeCell ref="A14:F14"/>
     <mergeCell ref="A17:F17"/>
@@ -4519,13 +4554,6 @@
     <mergeCell ref="A15:F15"/>
     <mergeCell ref="A12:F12"/>
     <mergeCell ref="A13:F13"/>
-    <mergeCell ref="A18:F18"/>
-    <mergeCell ref="C3:C6"/>
-    <mergeCell ref="D3:E6"/>
-    <mergeCell ref="F7:H9"/>
-    <mergeCell ref="C9:E9"/>
-    <mergeCell ref="A10:F10"/>
-    <mergeCell ref="A11:F11"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -4547,31 +4575,31 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="61.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="64" t="s">
+      <c r="A1" s="106" t="s">
         <v>54</v>
       </c>
-      <c r="B1" s="64"/>
-      <c r="C1" s="64"/>
-      <c r="D1" s="64"/>
-      <c r="E1" s="64"/>
-      <c r="F1" s="64"/>
-      <c r="G1" s="64"/>
-      <c r="H1" s="64"/>
-      <c r="I1" s="64"/>
-      <c r="J1" s="64"/>
-      <c r="K1" s="64"/>
-      <c r="L1" s="64"/>
+      <c r="B1" s="106"/>
+      <c r="C1" s="106"/>
+      <c r="D1" s="106"/>
+      <c r="E1" s="106"/>
+      <c r="F1" s="106"/>
+      <c r="G1" s="106"/>
+      <c r="H1" s="106"/>
+      <c r="I1" s="106"/>
+      <c r="J1" s="106"/>
+      <c r="K1" s="106"/>
+      <c r="L1" s="106"/>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="C3" s="65">
+      <c r="C3" s="107">
         <f>D3*C8</f>
         <v>0.67999999999999994</v>
       </c>
-      <c r="D3" s="66">
+      <c r="D3" s="108">
         <f>I20*10</f>
         <v>6.7999999999999989</v>
       </c>
-      <c r="E3" s="67"/>
+      <c r="E3" s="109"/>
       <c r="F3" s="11" t="s">
         <v>1</v>
       </c>
@@ -4598,9 +4626,9 @@
       </c>
     </row>
     <row r="4" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C4" s="65"/>
-      <c r="D4" s="66"/>
-      <c r="E4" s="67"/>
+      <c r="C4" s="107"/>
+      <c r="D4" s="108"/>
+      <c r="E4" s="109"/>
       <c r="F4" s="12" t="s">
         <v>4</v>
       </c>
@@ -4627,9 +4655,9 @@
       </c>
     </row>
     <row r="5" spans="1:15" ht="21" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C5" s="65"/>
-      <c r="D5" s="66"/>
-      <c r="E5" s="67"/>
+      <c r="C5" s="107"/>
+      <c r="D5" s="108"/>
+      <c r="E5" s="109"/>
       <c r="F5" s="13" t="s">
         <v>5</v>
       </c>
@@ -4656,9 +4684,9 @@
       </c>
     </row>
     <row r="6" spans="1:15" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C6" s="65"/>
-      <c r="D6" s="66"/>
-      <c r="E6" s="67"/>
+      <c r="C6" s="107"/>
+      <c r="D6" s="108"/>
+      <c r="E6" s="109"/>
       <c r="F6" s="13" t="s">
         <v>6</v>
       </c>
@@ -4685,12 +4713,12 @@
       </c>
     </row>
     <row r="7" spans="1:15" ht="24.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="F7" s="59" t="e" vm="1">
+      <c r="F7" s="110" t="e" vm="1">
         <f>_xlfn.XLOOKUP(H20,G4:G6,H4:H6,,-1)</f>
         <v>#VALUE!</v>
       </c>
-      <c r="G7" s="59"/>
-      <c r="H7" s="59"/>
+      <c r="G7" s="110"/>
+      <c r="H7" s="110"/>
       <c r="J7" s="10" t="s">
         <v>40</v>
       </c>
@@ -4714,9 +4742,9 @@
       <c r="C8" s="15">
         <v>0.1</v>
       </c>
-      <c r="F8" s="59"/>
-      <c r="G8" s="59"/>
-      <c r="H8" s="59"/>
+      <c r="F8" s="110"/>
+      <c r="G8" s="110"/>
+      <c r="H8" s="110"/>
       <c r="J8" s="7" t="s">
         <v>14</v>
       </c>
@@ -4734,14 +4762,14 @@
       </c>
     </row>
     <row r="9" spans="1:15" ht="70.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C9" s="60" t="s">
+      <c r="C9" s="111" t="s">
         <v>34</v>
       </c>
-      <c r="D9" s="60"/>
-      <c r="E9" s="60"/>
-      <c r="F9" s="59"/>
-      <c r="G9" s="59"/>
-      <c r="H9" s="59"/>
+      <c r="D9" s="111"/>
+      <c r="E9" s="111"/>
+      <c r="F9" s="110"/>
+      <c r="G9" s="110"/>
+      <c r="H9" s="110"/>
       <c r="J9" s="19" t="s">
         <v>39</v>
       </c>
@@ -4759,14 +4787,14 @@
       </c>
     </row>
     <row r="10" spans="1:15" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="68" t="s">
+      <c r="A10" s="113" t="s">
         <v>15</v>
       </c>
-      <c r="B10" s="68"/>
-      <c r="C10" s="68"/>
-      <c r="D10" s="68"/>
-      <c r="E10" s="68"/>
-      <c r="F10" s="69"/>
+      <c r="B10" s="113"/>
+      <c r="C10" s="113"/>
+      <c r="D10" s="113"/>
+      <c r="E10" s="113"/>
+      <c r="F10" s="114"/>
       <c r="G10" s="6" t="s">
         <v>7</v>
       </c>
@@ -4796,14 +4824,14 @@
       </c>
     </row>
     <row r="11" spans="1:15" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="63" t="s">
+      <c r="A11" s="112" t="s">
         <v>98</v>
       </c>
-      <c r="B11" s="63"/>
-      <c r="C11" s="63"/>
-      <c r="D11" s="63"/>
-      <c r="E11" s="63"/>
-      <c r="F11" s="63"/>
+      <c r="B11" s="112"/>
+      <c r="C11" s="112"/>
+      <c r="D11" s="112"/>
+      <c r="E11" s="112"/>
+      <c r="F11" s="112"/>
       <c r="G11" s="22">
         <v>0.1</v>
       </c>
@@ -4828,14 +4856,14 @@
       <c r="N11" s="31"/>
     </row>
     <row r="12" spans="1:15" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="63" t="s">
+      <c r="A12" s="112" t="s">
         <v>99</v>
       </c>
-      <c r="B12" s="63"/>
-      <c r="C12" s="63"/>
-      <c r="D12" s="63"/>
-      <c r="E12" s="63"/>
-      <c r="F12" s="63"/>
+      <c r="B12" s="112"/>
+      <c r="C12" s="112"/>
+      <c r="D12" s="112"/>
+      <c r="E12" s="112"/>
+      <c r="F12" s="112"/>
       <c r="G12" s="22">
         <v>0.1</v>
       </c>
@@ -4860,14 +4888,14 @@
       <c r="N12" s="31"/>
     </row>
     <row r="13" spans="1:15" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="63" t="s">
+      <c r="A13" s="112" t="s">
         <v>100</v>
       </c>
-      <c r="B13" s="63"/>
-      <c r="C13" s="63"/>
-      <c r="D13" s="63"/>
-      <c r="E13" s="63"/>
-      <c r="F13" s="63"/>
+      <c r="B13" s="112"/>
+      <c r="C13" s="112"/>
+      <c r="D13" s="112"/>
+      <c r="E13" s="112"/>
+      <c r="F13" s="112"/>
       <c r="G13" s="22">
         <v>0.1</v>
       </c>
@@ -4892,14 +4920,14 @@
       <c r="N13" s="31"/>
     </row>
     <row r="14" spans="1:15" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="63" t="s">
+      <c r="A14" s="112" t="s">
         <v>101</v>
       </c>
-      <c r="B14" s="63"/>
-      <c r="C14" s="63"/>
-      <c r="D14" s="63"/>
-      <c r="E14" s="63"/>
-      <c r="F14" s="63"/>
+      <c r="B14" s="112"/>
+      <c r="C14" s="112"/>
+      <c r="D14" s="112"/>
+      <c r="E14" s="112"/>
+      <c r="F14" s="112"/>
       <c r="G14" s="22">
         <v>0.15</v>
       </c>
@@ -4924,14 +4952,14 @@
       <c r="N14" s="31"/>
     </row>
     <row r="15" spans="1:15" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="63" t="s">
+      <c r="A15" s="112" t="s">
         <v>102</v>
       </c>
-      <c r="B15" s="63"/>
-      <c r="C15" s="63"/>
-      <c r="D15" s="63"/>
-      <c r="E15" s="63"/>
-      <c r="F15" s="63"/>
+      <c r="B15" s="112"/>
+      <c r="C15" s="112"/>
+      <c r="D15" s="112"/>
+      <c r="E15" s="112"/>
+      <c r="F15" s="112"/>
       <c r="G15" s="22">
         <v>0.1</v>
       </c>
@@ -4956,14 +4984,14 @@
       <c r="N15" s="31"/>
     </row>
     <row r="16" spans="1:15" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="63" t="s">
+      <c r="A16" s="112" t="s">
         <v>103</v>
       </c>
-      <c r="B16" s="63"/>
-      <c r="C16" s="63"/>
-      <c r="D16" s="63"/>
-      <c r="E16" s="63"/>
-      <c r="F16" s="63"/>
+      <c r="B16" s="112"/>
+      <c r="C16" s="112"/>
+      <c r="D16" s="112"/>
+      <c r="E16" s="112"/>
+      <c r="F16" s="112"/>
       <c r="G16" s="22">
         <v>0.1</v>
       </c>
@@ -4988,14 +5016,14 @@
       <c r="N16" s="31"/>
     </row>
     <row r="17" spans="1:14" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="63" t="s">
+      <c r="A17" s="112" t="s">
         <v>104</v>
       </c>
-      <c r="B17" s="63"/>
-      <c r="C17" s="63"/>
-      <c r="D17" s="63"/>
-      <c r="E17" s="63"/>
-      <c r="F17" s="63"/>
+      <c r="B17" s="112"/>
+      <c r="C17" s="112"/>
+      <c r="D17" s="112"/>
+      <c r="E17" s="112"/>
+      <c r="F17" s="112"/>
       <c r="G17" s="22">
         <v>0.15</v>
       </c>
@@ -5020,14 +5048,14 @@
       <c r="N17" s="31"/>
     </row>
     <row r="18" spans="1:14" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="63" t="s">
+      <c r="A18" s="112" t="s">
         <v>105</v>
       </c>
-      <c r="B18" s="63"/>
-      <c r="C18" s="63"/>
-      <c r="D18" s="63"/>
-      <c r="E18" s="63"/>
-      <c r="F18" s="63"/>
+      <c r="B18" s="112"/>
+      <c r="C18" s="112"/>
+      <c r="D18" s="112"/>
+      <c r="E18" s="112"/>
+      <c r="F18" s="112"/>
       <c r="G18" s="22">
         <v>0.1</v>
       </c>
@@ -5052,14 +5080,14 @@
       <c r="N18" s="31"/>
     </row>
     <row r="19" spans="1:14" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="63" t="s">
+      <c r="A19" s="112" t="s">
         <v>106</v>
       </c>
-      <c r="B19" s="63"/>
-      <c r="C19" s="63"/>
-      <c r="D19" s="63"/>
-      <c r="E19" s="63"/>
-      <c r="F19" s="63"/>
+      <c r="B19" s="112"/>
+      <c r="C19" s="112"/>
+      <c r="D19" s="112"/>
+      <c r="E19" s="112"/>
+      <c r="F19" s="112"/>
       <c r="G19" s="22">
         <v>0.1</v>
       </c>
@@ -5153,31 +5181,31 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="61.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="64" t="s">
+      <c r="A1" s="106" t="s">
         <v>55</v>
       </c>
-      <c r="B1" s="64"/>
-      <c r="C1" s="64"/>
-      <c r="D1" s="64"/>
-      <c r="E1" s="64"/>
-      <c r="F1" s="64"/>
-      <c r="G1" s="64"/>
-      <c r="H1" s="64"/>
-      <c r="I1" s="64"/>
-      <c r="J1" s="64"/>
-      <c r="K1" s="64"/>
-      <c r="L1" s="64"/>
+      <c r="B1" s="106"/>
+      <c r="C1" s="106"/>
+      <c r="D1" s="106"/>
+      <c r="E1" s="106"/>
+      <c r="F1" s="106"/>
+      <c r="G1" s="106"/>
+      <c r="H1" s="106"/>
+      <c r="I1" s="106"/>
+      <c r="J1" s="106"/>
+      <c r="K1" s="106"/>
+      <c r="L1" s="106"/>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="C3" s="65">
+      <c r="C3" s="107">
         <f>D3*C8</f>
         <v>0</v>
       </c>
-      <c r="D3" s="66">
+      <c r="D3" s="108">
         <f>I19*10</f>
         <v>0</v>
       </c>
-      <c r="E3" s="67"/>
+      <c r="E3" s="109"/>
       <c r="F3" s="11" t="s">
         <v>1</v>
       </c>
@@ -5204,9 +5232,9 @@
       </c>
     </row>
     <row r="4" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C4" s="65"/>
-      <c r="D4" s="66"/>
-      <c r="E4" s="67"/>
+      <c r="C4" s="107"/>
+      <c r="D4" s="108"/>
+      <c r="E4" s="109"/>
       <c r="F4" s="12" t="s">
         <v>4</v>
       </c>
@@ -5233,9 +5261,9 @@
       </c>
     </row>
     <row r="5" spans="1:15" ht="21" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C5" s="65"/>
-      <c r="D5" s="66"/>
-      <c r="E5" s="67"/>
+      <c r="C5" s="107"/>
+      <c r="D5" s="108"/>
+      <c r="E5" s="109"/>
       <c r="F5" s="13" t="s">
         <v>5</v>
       </c>
@@ -5262,9 +5290,9 @@
       </c>
     </row>
     <row r="6" spans="1:15" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C6" s="65"/>
-      <c r="D6" s="66"/>
-      <c r="E6" s="67"/>
+      <c r="C6" s="107"/>
+      <c r="D6" s="108"/>
+      <c r="E6" s="109"/>
       <c r="F6" s="13" t="s">
         <v>6</v>
       </c>
@@ -5291,12 +5319,12 @@
       </c>
     </row>
     <row r="7" spans="1:15" ht="24.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="F7" s="59" t="e" vm="5">
+      <c r="F7" s="110" t="e" vm="6">
         <f>_xlfn.XLOOKUP(H19,G4:G6,H4:H6,,-1)</f>
         <v>#VALUE!</v>
       </c>
-      <c r="G7" s="59"/>
-      <c r="H7" s="59"/>
+      <c r="G7" s="110"/>
+      <c r="H7" s="110"/>
       <c r="J7" s="10" t="s">
         <v>40</v>
       </c>
@@ -5320,9 +5348,9 @@
       <c r="C8" s="15">
         <v>0.2</v>
       </c>
-      <c r="F8" s="59"/>
-      <c r="G8" s="59"/>
-      <c r="H8" s="59"/>
+      <c r="F8" s="110"/>
+      <c r="G8" s="110"/>
+      <c r="H8" s="110"/>
       <c r="J8" s="7" t="s">
         <v>14</v>
       </c>
@@ -5340,14 +5368,14 @@
       </c>
     </row>
     <row r="9" spans="1:15" ht="70.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C9" s="60" t="s">
+      <c r="C9" s="111" t="s">
         <v>35</v>
       </c>
-      <c r="D9" s="60"/>
-      <c r="E9" s="60"/>
-      <c r="F9" s="59"/>
-      <c r="G9" s="59"/>
-      <c r="H9" s="59"/>
+      <c r="D9" s="111"/>
+      <c r="E9" s="111"/>
+      <c r="F9" s="110"/>
+      <c r="G9" s="110"/>
+      <c r="H9" s="110"/>
       <c r="J9" s="19" t="s">
         <v>39</v>
       </c>
@@ -5365,14 +5393,14 @@
       </c>
     </row>
     <row r="10" spans="1:15" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="68" t="s">
+      <c r="A10" s="113" t="s">
         <v>15</v>
       </c>
-      <c r="B10" s="68"/>
-      <c r="C10" s="68"/>
-      <c r="D10" s="68"/>
-      <c r="E10" s="68"/>
-      <c r="F10" s="69"/>
+      <c r="B10" s="113"/>
+      <c r="C10" s="113"/>
+      <c r="D10" s="113"/>
+      <c r="E10" s="113"/>
+      <c r="F10" s="114"/>
       <c r="G10" s="6" t="s">
         <v>7</v>
       </c>
@@ -5402,14 +5430,14 @@
       </c>
     </row>
     <row r="11" spans="1:15" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="63" t="s">
+      <c r="A11" s="112" t="s">
         <v>90</v>
       </c>
-      <c r="B11" s="63"/>
-      <c r="C11" s="63"/>
-      <c r="D11" s="63"/>
-      <c r="E11" s="63"/>
-      <c r="F11" s="63"/>
+      <c r="B11" s="112"/>
+      <c r="C11" s="112"/>
+      <c r="D11" s="112"/>
+      <c r="E11" s="112"/>
+      <c r="F11" s="112"/>
       <c r="G11" s="22">
         <v>0.15</v>
       </c>
@@ -5434,14 +5462,14 @@
       </c>
     </row>
     <row r="12" spans="1:15" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="63" t="s">
+      <c r="A12" s="112" t="s">
         <v>91</v>
       </c>
-      <c r="B12" s="63"/>
-      <c r="C12" s="63"/>
-      <c r="D12" s="63"/>
-      <c r="E12" s="63"/>
-      <c r="F12" s="63"/>
+      <c r="B12" s="112"/>
+      <c r="C12" s="112"/>
+      <c r="D12" s="112"/>
+      <c r="E12" s="112"/>
+      <c r="F12" s="112"/>
       <c r="G12" s="22">
         <v>0.1</v>
       </c>
@@ -5466,14 +5494,14 @@
       </c>
     </row>
     <row r="13" spans="1:15" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="63" t="s">
+      <c r="A13" s="112" t="s">
         <v>92</v>
       </c>
-      <c r="B13" s="63"/>
-      <c r="C13" s="63"/>
-      <c r="D13" s="63"/>
-      <c r="E13" s="63"/>
-      <c r="F13" s="63"/>
+      <c r="B13" s="112"/>
+      <c r="C13" s="112"/>
+      <c r="D13" s="112"/>
+      <c r="E13" s="112"/>
+      <c r="F13" s="112"/>
       <c r="G13" s="22">
         <v>0.1</v>
       </c>
@@ -5498,14 +5526,14 @@
       </c>
     </row>
     <row r="14" spans="1:15" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="63" t="s">
+      <c r="A14" s="112" t="s">
         <v>93</v>
       </c>
-      <c r="B14" s="63"/>
-      <c r="C14" s="63"/>
-      <c r="D14" s="63"/>
-      <c r="E14" s="63"/>
-      <c r="F14" s="63"/>
+      <c r="B14" s="112"/>
+      <c r="C14" s="112"/>
+      <c r="D14" s="112"/>
+      <c r="E14" s="112"/>
+      <c r="F14" s="112"/>
       <c r="G14" s="22">
         <v>0.15</v>
       </c>
@@ -5530,14 +5558,14 @@
       </c>
     </row>
     <row r="15" spans="1:15" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="63" t="s">
+      <c r="A15" s="112" t="s">
         <v>94</v>
       </c>
-      <c r="B15" s="63"/>
-      <c r="C15" s="63"/>
-      <c r="D15" s="63"/>
-      <c r="E15" s="63"/>
-      <c r="F15" s="63"/>
+      <c r="B15" s="112"/>
+      <c r="C15" s="112"/>
+      <c r="D15" s="112"/>
+      <c r="E15" s="112"/>
+      <c r="F15" s="112"/>
       <c r="G15" s="22">
         <v>0.1</v>
       </c>
@@ -5562,14 +5590,14 @@
       </c>
     </row>
     <row r="16" spans="1:15" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="63" t="s">
+      <c r="A16" s="112" t="s">
         <v>95</v>
       </c>
-      <c r="B16" s="63"/>
-      <c r="C16" s="63"/>
-      <c r="D16" s="63"/>
-      <c r="E16" s="63"/>
-      <c r="F16" s="63"/>
+      <c r="B16" s="112"/>
+      <c r="C16" s="112"/>
+      <c r="D16" s="112"/>
+      <c r="E16" s="112"/>
+      <c r="F16" s="112"/>
       <c r="G16" s="22">
         <v>0.15</v>
       </c>
@@ -5594,14 +5622,14 @@
       </c>
     </row>
     <row r="17" spans="1:14" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="63" t="s">
+      <c r="A17" s="112" t="s">
         <v>96</v>
       </c>
-      <c r="B17" s="63"/>
-      <c r="C17" s="63"/>
-      <c r="D17" s="63"/>
-      <c r="E17" s="63"/>
-      <c r="F17" s="63"/>
+      <c r="B17" s="112"/>
+      <c r="C17" s="112"/>
+      <c r="D17" s="112"/>
+      <c r="E17" s="112"/>
+      <c r="F17" s="112"/>
       <c r="G17" s="22">
         <v>0.15</v>
       </c>
@@ -5626,14 +5654,14 @@
       </c>
     </row>
     <row r="18" spans="1:14" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="63" t="s">
+      <c r="A18" s="112" t="s">
         <v>97</v>
       </c>
-      <c r="B18" s="63"/>
-      <c r="C18" s="63"/>
-      <c r="D18" s="63"/>
-      <c r="E18" s="63"/>
-      <c r="F18" s="63"/>
+      <c r="B18" s="112"/>
+      <c r="C18" s="112"/>
+      <c r="D18" s="112"/>
+      <c r="E18" s="112"/>
+      <c r="F18" s="112"/>
       <c r="G18" s="22">
         <v>0.1</v>
       </c>
@@ -5691,12 +5719,6 @@
     </row>
   </sheetData>
   <mergeCells count="14">
-    <mergeCell ref="A16:F16"/>
-    <mergeCell ref="A17:F17"/>
-    <mergeCell ref="A18:F18"/>
-    <mergeCell ref="A12:F12"/>
-    <mergeCell ref="A13:F13"/>
-    <mergeCell ref="A14:F14"/>
     <mergeCell ref="A1:L1"/>
     <mergeCell ref="A11:F11"/>
     <mergeCell ref="A15:F15"/>
@@ -5705,6 +5727,12 @@
     <mergeCell ref="F7:H9"/>
     <mergeCell ref="C9:E9"/>
     <mergeCell ref="A10:F10"/>
+    <mergeCell ref="A16:F16"/>
+    <mergeCell ref="A17:F17"/>
+    <mergeCell ref="A18:F18"/>
+    <mergeCell ref="A12:F12"/>
+    <mergeCell ref="A13:F13"/>
+    <mergeCell ref="A14:F14"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -5726,31 +5754,31 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="61.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="64" t="s">
+      <c r="A1" s="106" t="s">
         <v>56</v>
       </c>
-      <c r="B1" s="64"/>
-      <c r="C1" s="64"/>
-      <c r="D1" s="64"/>
-      <c r="E1" s="64"/>
-      <c r="F1" s="64"/>
-      <c r="G1" s="64"/>
-      <c r="H1" s="64"/>
-      <c r="I1" s="64"/>
-      <c r="J1" s="64"/>
-      <c r="K1" s="64"/>
-      <c r="L1" s="64"/>
+      <c r="B1" s="106"/>
+      <c r="C1" s="106"/>
+      <c r="D1" s="106"/>
+      <c r="E1" s="106"/>
+      <c r="F1" s="106"/>
+      <c r="G1" s="106"/>
+      <c r="H1" s="106"/>
+      <c r="I1" s="106"/>
+      <c r="J1" s="106"/>
+      <c r="K1" s="106"/>
+      <c r="L1" s="106"/>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="C3" s="65">
+      <c r="C3" s="107">
         <f>D3*C8</f>
         <v>0</v>
       </c>
-      <c r="D3" s="66">
+      <c r="D3" s="108">
         <f>I19*10</f>
         <v>0</v>
       </c>
-      <c r="E3" s="67"/>
+      <c r="E3" s="109"/>
       <c r="F3" s="11" t="s">
         <v>1</v>
       </c>
@@ -5777,9 +5805,9 @@
       </c>
     </row>
     <row r="4" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C4" s="65"/>
-      <c r="D4" s="66"/>
-      <c r="E4" s="67"/>
+      <c r="C4" s="107"/>
+      <c r="D4" s="108"/>
+      <c r="E4" s="109"/>
       <c r="F4" s="12" t="s">
         <v>4</v>
       </c>
@@ -5806,9 +5834,9 @@
       </c>
     </row>
     <row r="5" spans="1:15" ht="21" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C5" s="65"/>
-      <c r="D5" s="66"/>
-      <c r="E5" s="67"/>
+      <c r="C5" s="107"/>
+      <c r="D5" s="108"/>
+      <c r="E5" s="109"/>
       <c r="F5" s="13" t="s">
         <v>5</v>
       </c>
@@ -5835,9 +5863,9 @@
       </c>
     </row>
     <row r="6" spans="1:15" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C6" s="65"/>
-      <c r="D6" s="66"/>
-      <c r="E6" s="67"/>
+      <c r="C6" s="107"/>
+      <c r="D6" s="108"/>
+      <c r="E6" s="109"/>
       <c r="F6" s="13" t="s">
         <v>6</v>
       </c>
@@ -5864,12 +5892,12 @@
       </c>
     </row>
     <row r="7" spans="1:15" ht="24.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="F7" s="59" t="e" vm="5">
+      <c r="F7" s="110" t="e" vm="6">
         <f>_xlfn.XLOOKUP(H19,G4:G6,H4:H6,,-1)</f>
         <v>#VALUE!</v>
       </c>
-      <c r="G7" s="59"/>
-      <c r="H7" s="59"/>
+      <c r="G7" s="110"/>
+      <c r="H7" s="110"/>
       <c r="J7" s="10" t="s">
         <v>40</v>
       </c>
@@ -5893,9 +5921,9 @@
       <c r="C8" s="15">
         <v>0.05</v>
       </c>
-      <c r="F8" s="59"/>
-      <c r="G8" s="59"/>
-      <c r="H8" s="59"/>
+      <c r="F8" s="110"/>
+      <c r="G8" s="110"/>
+      <c r="H8" s="110"/>
       <c r="J8" s="7" t="s">
         <v>14</v>
       </c>
@@ -5913,14 +5941,14 @@
       </c>
     </row>
     <row r="9" spans="1:15" ht="70.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C9" s="60" t="s">
+      <c r="C9" s="111" t="s">
         <v>36</v>
       </c>
-      <c r="D9" s="60"/>
-      <c r="E9" s="60"/>
-      <c r="F9" s="59"/>
-      <c r="G9" s="59"/>
-      <c r="H9" s="59"/>
+      <c r="D9" s="111"/>
+      <c r="E9" s="111"/>
+      <c r="F9" s="110"/>
+      <c r="G9" s="110"/>
+      <c r="H9" s="110"/>
       <c r="J9" s="19" t="s">
         <v>39</v>
       </c>
@@ -5938,14 +5966,14 @@
       </c>
     </row>
     <row r="10" spans="1:15" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="68" t="s">
+      <c r="A10" s="113" t="s">
         <v>15</v>
       </c>
-      <c r="B10" s="68"/>
-      <c r="C10" s="68"/>
-      <c r="D10" s="68"/>
-      <c r="E10" s="68"/>
-      <c r="F10" s="69"/>
+      <c r="B10" s="113"/>
+      <c r="C10" s="113"/>
+      <c r="D10" s="113"/>
+      <c r="E10" s="113"/>
+      <c r="F10" s="114"/>
       <c r="G10" s="6" t="s">
         <v>7</v>
       </c>
@@ -5975,14 +6003,14 @@
       </c>
     </row>
     <row r="11" spans="1:15" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="63" t="s">
+      <c r="A11" s="112" t="s">
         <v>82</v>
       </c>
-      <c r="B11" s="63"/>
-      <c r="C11" s="63"/>
-      <c r="D11" s="63"/>
-      <c r="E11" s="63"/>
-      <c r="F11" s="63"/>
+      <c r="B11" s="112"/>
+      <c r="C11" s="112"/>
+      <c r="D11" s="112"/>
+      <c r="E11" s="112"/>
+      <c r="F11" s="112"/>
       <c r="G11" s="22">
         <v>0.15</v>
       </c>
@@ -6004,14 +6032,14 @@
       <c r="N11" s="31"/>
     </row>
     <row r="12" spans="1:15" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="63" t="s">
+      <c r="A12" s="112" t="s">
         <v>83</v>
       </c>
-      <c r="B12" s="63"/>
-      <c r="C12" s="63"/>
-      <c r="D12" s="63"/>
-      <c r="E12" s="63"/>
-      <c r="F12" s="63"/>
+      <c r="B12" s="112"/>
+      <c r="C12" s="112"/>
+      <c r="D12" s="112"/>
+      <c r="E12" s="112"/>
+      <c r="F12" s="112"/>
       <c r="G12" s="22">
         <v>0.15</v>
       </c>
@@ -6033,14 +6061,14 @@
       <c r="N12" s="31"/>
     </row>
     <row r="13" spans="1:15" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="63" t="s">
+      <c r="A13" s="112" t="s">
         <v>84</v>
       </c>
-      <c r="B13" s="63"/>
-      <c r="C13" s="63"/>
-      <c r="D13" s="63"/>
-      <c r="E13" s="63"/>
-      <c r="F13" s="63"/>
+      <c r="B13" s="112"/>
+      <c r="C13" s="112"/>
+      <c r="D13" s="112"/>
+      <c r="E13" s="112"/>
+      <c r="F13" s="112"/>
       <c r="G13" s="22">
         <v>0.1</v>
       </c>
@@ -6062,14 +6090,14 @@
       <c r="N13" s="31"/>
     </row>
     <row r="14" spans="1:15" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="63" t="s">
+      <c r="A14" s="112" t="s">
         <v>85</v>
       </c>
-      <c r="B14" s="63"/>
-      <c r="C14" s="63"/>
-      <c r="D14" s="63"/>
-      <c r="E14" s="63"/>
-      <c r="F14" s="63"/>
+      <c r="B14" s="112"/>
+      <c r="C14" s="112"/>
+      <c r="D14" s="112"/>
+      <c r="E14" s="112"/>
+      <c r="F14" s="112"/>
       <c r="G14" s="22">
         <v>0.15</v>
       </c>
@@ -6091,14 +6119,14 @@
       <c r="N14" s="31"/>
     </row>
     <row r="15" spans="1:15" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="63" t="s">
+      <c r="A15" s="112" t="s">
         <v>86</v>
       </c>
-      <c r="B15" s="63"/>
-      <c r="C15" s="63"/>
-      <c r="D15" s="63"/>
-      <c r="E15" s="63"/>
-      <c r="F15" s="63"/>
+      <c r="B15" s="112"/>
+      <c r="C15" s="112"/>
+      <c r="D15" s="112"/>
+      <c r="E15" s="112"/>
+      <c r="F15" s="112"/>
       <c r="G15" s="22">
         <v>0.1</v>
       </c>
@@ -6120,14 +6148,14 @@
       <c r="N15" s="31"/>
     </row>
     <row r="16" spans="1:15" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="63" t="s">
+      <c r="A16" s="112" t="s">
         <v>87</v>
       </c>
-      <c r="B16" s="63"/>
-      <c r="C16" s="63"/>
-      <c r="D16" s="63"/>
-      <c r="E16" s="63"/>
-      <c r="F16" s="63"/>
+      <c r="B16" s="112"/>
+      <c r="C16" s="112"/>
+      <c r="D16" s="112"/>
+      <c r="E16" s="112"/>
+      <c r="F16" s="112"/>
       <c r="G16" s="22">
         <v>0.1</v>
       </c>
@@ -6149,14 +6177,14 @@
       <c r="N16" s="31"/>
     </row>
     <row r="17" spans="1:14" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="63" t="s">
+      <c r="A17" s="112" t="s">
         <v>88</v>
       </c>
-      <c r="B17" s="63"/>
-      <c r="C17" s="63"/>
-      <c r="D17" s="63"/>
-      <c r="E17" s="63"/>
-      <c r="F17" s="63"/>
+      <c r="B17" s="112"/>
+      <c r="C17" s="112"/>
+      <c r="D17" s="112"/>
+      <c r="E17" s="112"/>
+      <c r="F17" s="112"/>
       <c r="G17" s="22">
         <v>0.15</v>
       </c>
@@ -6178,14 +6206,14 @@
       <c r="N17" s="31"/>
     </row>
     <row r="18" spans="1:14" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="63" t="s">
+      <c r="A18" s="112" t="s">
         <v>89</v>
       </c>
-      <c r="B18" s="63"/>
-      <c r="C18" s="63"/>
-      <c r="D18" s="63"/>
-      <c r="E18" s="63"/>
-      <c r="F18" s="63"/>
+      <c r="B18" s="112"/>
+      <c r="C18" s="112"/>
+      <c r="D18" s="112"/>
+      <c r="E18" s="112"/>
+      <c r="F18" s="112"/>
       <c r="G18" s="22">
         <v>0.1</v>
       </c>
@@ -6240,12 +6268,6 @@
     </row>
   </sheetData>
   <mergeCells count="14">
-    <mergeCell ref="A16:F16"/>
-    <mergeCell ref="A17:F17"/>
-    <mergeCell ref="A18:F18"/>
-    <mergeCell ref="A12:F12"/>
-    <mergeCell ref="A13:F13"/>
-    <mergeCell ref="A14:F14"/>
     <mergeCell ref="A1:L1"/>
     <mergeCell ref="A11:F11"/>
     <mergeCell ref="A15:F15"/>
@@ -6254,6 +6276,12 @@
     <mergeCell ref="F7:H9"/>
     <mergeCell ref="C9:E9"/>
     <mergeCell ref="A10:F10"/>
+    <mergeCell ref="A16:F16"/>
+    <mergeCell ref="A17:F17"/>
+    <mergeCell ref="A18:F18"/>
+    <mergeCell ref="A12:F12"/>
+    <mergeCell ref="A13:F13"/>
+    <mergeCell ref="A14:F14"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -6275,31 +6303,31 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="61.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="64" t="s">
+      <c r="A1" s="106" t="s">
         <v>57</v>
       </c>
-      <c r="B1" s="64"/>
-      <c r="C1" s="64"/>
-      <c r="D1" s="64"/>
-      <c r="E1" s="64"/>
-      <c r="F1" s="64"/>
-      <c r="G1" s="64"/>
-      <c r="H1" s="64"/>
-      <c r="I1" s="64"/>
-      <c r="J1" s="64"/>
-      <c r="K1" s="64"/>
-      <c r="L1" s="64"/>
+      <c r="B1" s="106"/>
+      <c r="C1" s="106"/>
+      <c r="D1" s="106"/>
+      <c r="E1" s="106"/>
+      <c r="F1" s="106"/>
+      <c r="G1" s="106"/>
+      <c r="H1" s="106"/>
+      <c r="I1" s="106"/>
+      <c r="J1" s="106"/>
+      <c r="K1" s="106"/>
+      <c r="L1" s="106"/>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="C3" s="65">
+      <c r="C3" s="107">
         <f>D3*C8</f>
         <v>1.3599999999999999</v>
       </c>
-      <c r="D3" s="66">
+      <c r="D3" s="108">
         <f>I20*10</f>
         <v>6.7999999999999989</v>
       </c>
-      <c r="E3" s="67"/>
+      <c r="E3" s="109"/>
       <c r="F3" s="11" t="s">
         <v>1</v>
       </c>
@@ -6326,9 +6354,9 @@
       </c>
     </row>
     <row r="4" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C4" s="65"/>
-      <c r="D4" s="66"/>
-      <c r="E4" s="67"/>
+      <c r="C4" s="107"/>
+      <c r="D4" s="108"/>
+      <c r="E4" s="109"/>
       <c r="F4" s="12" t="s">
         <v>4</v>
       </c>
@@ -6355,9 +6383,9 @@
       </c>
     </row>
     <row r="5" spans="1:15" ht="21" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C5" s="65"/>
-      <c r="D5" s="66"/>
-      <c r="E5" s="67"/>
+      <c r="C5" s="107"/>
+      <c r="D5" s="108"/>
+      <c r="E5" s="109"/>
       <c r="F5" s="13" t="s">
         <v>5</v>
       </c>
@@ -6384,9 +6412,9 @@
       </c>
     </row>
     <row r="6" spans="1:15" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C6" s="65"/>
-      <c r="D6" s="66"/>
-      <c r="E6" s="67"/>
+      <c r="C6" s="107"/>
+      <c r="D6" s="108"/>
+      <c r="E6" s="109"/>
       <c r="F6" s="13" t="s">
         <v>6</v>
       </c>
@@ -6413,12 +6441,12 @@
       </c>
     </row>
     <row r="7" spans="1:15" ht="24.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="F7" s="59" t="e" vm="1">
+      <c r="F7" s="110" t="e" vm="1">
         <f>_xlfn.XLOOKUP(H20,G4:G6,H4:H6,,-1)</f>
         <v>#VALUE!</v>
       </c>
-      <c r="G7" s="59"/>
-      <c r="H7" s="59"/>
+      <c r="G7" s="110"/>
+      <c r="H7" s="110"/>
       <c r="J7" s="10" t="s">
         <v>40</v>
       </c>
@@ -6442,9 +6470,9 @@
       <c r="C8" s="15">
         <v>0.2</v>
       </c>
-      <c r="F8" s="59"/>
-      <c r="G8" s="59"/>
-      <c r="H8" s="59"/>
+      <c r="F8" s="110"/>
+      <c r="G8" s="110"/>
+      <c r="H8" s="110"/>
       <c r="J8" s="7" t="s">
         <v>14</v>
       </c>
@@ -6462,14 +6490,14 @@
       </c>
     </row>
     <row r="9" spans="1:15" ht="70.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C9" s="60" t="s">
+      <c r="C9" s="111" t="s">
         <v>37</v>
       </c>
-      <c r="D9" s="60"/>
-      <c r="E9" s="60"/>
-      <c r="F9" s="59"/>
-      <c r="G9" s="59"/>
-      <c r="H9" s="59"/>
+      <c r="D9" s="111"/>
+      <c r="E9" s="111"/>
+      <c r="F9" s="110"/>
+      <c r="G9" s="110"/>
+      <c r="H9" s="110"/>
       <c r="J9" s="19" t="s">
         <v>39</v>
       </c>
@@ -6487,14 +6515,14 @@
       </c>
     </row>
     <row r="10" spans="1:15" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="68" t="s">
+      <c r="A10" s="113" t="s">
         <v>15</v>
       </c>
-      <c r="B10" s="68"/>
-      <c r="C10" s="68"/>
-      <c r="D10" s="68"/>
-      <c r="E10" s="68"/>
-      <c r="F10" s="69"/>
+      <c r="B10" s="113"/>
+      <c r="C10" s="113"/>
+      <c r="D10" s="113"/>
+      <c r="E10" s="113"/>
+      <c r="F10" s="114"/>
       <c r="G10" s="6" t="s">
         <v>7</v>
       </c>
@@ -6524,14 +6552,14 @@
       </c>
     </row>
     <row r="11" spans="1:15" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="63" t="s">
+      <c r="A11" s="112" t="s">
         <v>73</v>
       </c>
-      <c r="B11" s="63"/>
-      <c r="C11" s="63"/>
-      <c r="D11" s="63"/>
-      <c r="E11" s="63"/>
-      <c r="F11" s="63"/>
+      <c r="B11" s="112"/>
+      <c r="C11" s="112"/>
+      <c r="D11" s="112"/>
+      <c r="E11" s="112"/>
+      <c r="F11" s="112"/>
       <c r="G11" s="22">
         <v>0.15</v>
       </c>
@@ -6556,14 +6584,14 @@
       <c r="N11" s="31"/>
     </row>
     <row r="12" spans="1:15" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="63" t="s">
+      <c r="A12" s="112" t="s">
         <v>74</v>
       </c>
-      <c r="B12" s="63"/>
-      <c r="C12" s="63"/>
-      <c r="D12" s="63"/>
-      <c r="E12" s="63"/>
-      <c r="F12" s="63"/>
+      <c r="B12" s="112"/>
+      <c r="C12" s="112"/>
+      <c r="D12" s="112"/>
+      <c r="E12" s="112"/>
+      <c r="F12" s="112"/>
       <c r="G12" s="22">
         <v>0.1</v>
       </c>
@@ -6588,14 +6616,14 @@
       <c r="N12" s="31"/>
     </row>
     <row r="13" spans="1:15" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="63" t="s">
+      <c r="A13" s="112" t="s">
         <v>75</v>
       </c>
-      <c r="B13" s="63"/>
-      <c r="C13" s="63"/>
-      <c r="D13" s="63"/>
-      <c r="E13" s="63"/>
-      <c r="F13" s="63"/>
+      <c r="B13" s="112"/>
+      <c r="C13" s="112"/>
+      <c r="D13" s="112"/>
+      <c r="E13" s="112"/>
+      <c r="F13" s="112"/>
       <c r="G13" s="22">
         <v>0.1</v>
       </c>
@@ -6620,14 +6648,14 @@
       <c r="N13" s="31"/>
     </row>
     <row r="14" spans="1:15" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="63" t="s">
+      <c r="A14" s="112" t="s">
         <v>76</v>
       </c>
-      <c r="B14" s="63"/>
-      <c r="C14" s="63"/>
-      <c r="D14" s="63"/>
-      <c r="E14" s="63"/>
-      <c r="F14" s="63"/>
+      <c r="B14" s="112"/>
+      <c r="C14" s="112"/>
+      <c r="D14" s="112"/>
+      <c r="E14" s="112"/>
+      <c r="F14" s="112"/>
       <c r="G14" s="22">
         <v>0.15</v>
       </c>
@@ -6652,14 +6680,14 @@
       <c r="N14" s="31"/>
     </row>
     <row r="15" spans="1:15" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="63" t="s">
+      <c r="A15" s="112" t="s">
         <v>77</v>
       </c>
-      <c r="B15" s="63"/>
-      <c r="C15" s="63"/>
-      <c r="D15" s="63"/>
-      <c r="E15" s="63"/>
-      <c r="F15" s="63"/>
+      <c r="B15" s="112"/>
+      <c r="C15" s="112"/>
+      <c r="D15" s="112"/>
+      <c r="E15" s="112"/>
+      <c r="F15" s="112"/>
       <c r="G15" s="22">
         <v>0.1</v>
       </c>
@@ -6684,14 +6712,14 @@
       <c r="N15" s="31"/>
     </row>
     <row r="16" spans="1:15" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="63" t="s">
+      <c r="A16" s="112" t="s">
         <v>78</v>
       </c>
-      <c r="B16" s="63"/>
-      <c r="C16" s="63"/>
-      <c r="D16" s="63"/>
-      <c r="E16" s="63"/>
-      <c r="F16" s="63"/>
+      <c r="B16" s="112"/>
+      <c r="C16" s="112"/>
+      <c r="D16" s="112"/>
+      <c r="E16" s="112"/>
+      <c r="F16" s="112"/>
       <c r="G16" s="22">
         <v>0.1</v>
       </c>
@@ -6716,14 +6744,14 @@
       <c r="N16" s="31"/>
     </row>
     <row r="17" spans="1:14" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="63" t="s">
+      <c r="A17" s="112" t="s">
         <v>79</v>
       </c>
-      <c r="B17" s="63"/>
-      <c r="C17" s="63"/>
-      <c r="D17" s="63"/>
-      <c r="E17" s="63"/>
-      <c r="F17" s="63"/>
+      <c r="B17" s="112"/>
+      <c r="C17" s="112"/>
+      <c r="D17" s="112"/>
+      <c r="E17" s="112"/>
+      <c r="F17" s="112"/>
       <c r="G17" s="22">
         <v>0.1</v>
       </c>
@@ -6748,14 +6776,14 @@
       <c r="N17" s="31"/>
     </row>
     <row r="18" spans="1:14" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="63" t="s">
+      <c r="A18" s="112" t="s">
         <v>80</v>
       </c>
-      <c r="B18" s="63"/>
-      <c r="C18" s="63"/>
-      <c r="D18" s="63"/>
-      <c r="E18" s="63"/>
-      <c r="F18" s="63"/>
+      <c r="B18" s="112"/>
+      <c r="C18" s="112"/>
+      <c r="D18" s="112"/>
+      <c r="E18" s="112"/>
+      <c r="F18" s="112"/>
       <c r="G18" s="22">
         <v>0.1</v>
       </c>
@@ -6780,14 +6808,14 @@
       <c r="N18" s="31"/>
     </row>
     <row r="19" spans="1:14" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="63" t="s">
+      <c r="A19" s="112" t="s">
         <v>81</v>
       </c>
-      <c r="B19" s="63"/>
-      <c r="C19" s="63"/>
-      <c r="D19" s="63"/>
-      <c r="E19" s="63"/>
-      <c r="F19" s="63"/>
+      <c r="B19" s="112"/>
+      <c r="C19" s="112"/>
+      <c r="D19" s="112"/>
+      <c r="E19" s="112"/>
+      <c r="F19" s="112"/>
       <c r="G19" s="22">
         <v>0.1</v>
       </c>
@@ -6845,13 +6873,6 @@
     </row>
   </sheetData>
   <mergeCells count="15">
-    <mergeCell ref="A16:F16"/>
-    <mergeCell ref="A17:F17"/>
-    <mergeCell ref="A18:F18"/>
-    <mergeCell ref="A19:F19"/>
-    <mergeCell ref="A12:F12"/>
-    <mergeCell ref="A13:F13"/>
-    <mergeCell ref="A14:F14"/>
     <mergeCell ref="A1:L1"/>
     <mergeCell ref="A11:F11"/>
     <mergeCell ref="A15:F15"/>
@@ -6860,6 +6881,13 @@
     <mergeCell ref="F7:H9"/>
     <mergeCell ref="C9:E9"/>
     <mergeCell ref="A10:F10"/>
+    <mergeCell ref="A16:F16"/>
+    <mergeCell ref="A17:F17"/>
+    <mergeCell ref="A18:F18"/>
+    <mergeCell ref="A19:F19"/>
+    <mergeCell ref="A12:F12"/>
+    <mergeCell ref="A13:F13"/>
+    <mergeCell ref="A14:F14"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -6876,18 +6904,18 @@
     <col min="5" max="6" width="23.109375" customWidth="1"/>
     <col min="7" max="7" width="23" customWidth="1"/>
     <col min="8" max="8" width="23.109375" customWidth="1"/>
-    <col min="9" max="9" width="11.5546875" style="83"/>
+    <col min="9" max="9" width="11.5546875" style="60"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="74" t="s">
-        <v>141</v>
-      </c>
-      <c r="B1" s="77" t="s">
+      <c r="A1" s="115" t="s">
+        <v>287</v>
+      </c>
+      <c r="B1" s="118" t="s">
         <v>111</v>
       </c>
-      <c r="C1" s="79"/>
-      <c r="D1" s="72" t="s">
+      <c r="C1" s="124"/>
+      <c r="D1" s="122" t="s">
         <v>112</v>
       </c>
       <c r="E1" s="42" t="s">
@@ -6902,15 +6930,15 @@
       <c r="H1" s="42" t="s">
         <v>119</v>
       </c>
-      <c r="I1" s="70" t="s">
-        <v>146</v>
+      <c r="I1" s="120" t="s">
+        <v>145</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A2" s="75"/>
-      <c r="B2" s="78"/>
-      <c r="C2" s="80"/>
-      <c r="D2" s="73"/>
+      <c r="A2" s="116"/>
+      <c r="B2" s="119"/>
+      <c r="C2" s="125"/>
+      <c r="D2" s="123"/>
       <c r="E2" s="39" t="s">
         <v>114</v>
       </c>
@@ -6923,12 +6951,12 @@
       <c r="H2" s="39" t="s">
         <v>120</v>
       </c>
-      <c r="I2" s="71"/>
+      <c r="I2" s="121"/>
     </row>
     <row r="3" spans="1:9" ht="71.400000000000006" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="75"/>
+      <c r="A3" s="116"/>
       <c r="B3" s="56" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="C3" s="34">
         <v>0.4</v>
@@ -6953,9 +6981,9 @@
       </c>
     </row>
     <row r="4" spans="1:9" ht="72" x14ac:dyDescent="0.3">
-      <c r="A4" s="75"/>
+      <c r="A4" s="116"/>
       <c r="B4" s="56" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="C4" s="34">
         <v>0.3</v>
@@ -6980,9 +7008,9 @@
       </c>
     </row>
     <row r="5" spans="1:9" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A5" s="75"/>
+      <c r="A5" s="116"/>
       <c r="B5" s="56" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C5" s="34">
         <v>0.2</v>
@@ -7007,9 +7035,9 @@
       </c>
     </row>
     <row r="6" spans="1:9" ht="61.2" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="75"/>
+      <c r="A6" s="116"/>
       <c r="B6" s="57" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="C6" s="46">
         <v>0.1</v>
@@ -7034,9 +7062,9 @@
       </c>
     </row>
     <row r="7" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="76"/>
+      <c r="A7" s="117"/>
       <c r="B7" s="55" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="C7" s="37"/>
       <c r="D7" s="32"/>
@@ -7044,21 +7072,21 @@
       <c r="F7" s="32"/>
       <c r="G7" s="32"/>
       <c r="H7" s="38"/>
-      <c r="I7" s="82">
+      <c r="I7" s="59">
         <f>IF(COUNT(I3:I6)&gt;0,I3*C3+I4*C4+I5*C5+I6*C6,"")</f>
         <v>7.2000000000000011</v>
       </c>
     </row>
     <row r="8" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="9" spans="1:9" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="74" t="s">
-        <v>178</v>
-      </c>
-      <c r="B9" s="77" t="s">
+      <c r="A9" s="115" t="s">
+        <v>288</v>
+      </c>
+      <c r="B9" s="118" t="s">
         <v>111</v>
       </c>
-      <c r="C9" s="79"/>
-      <c r="D9" s="72" t="s">
+      <c r="C9" s="124"/>
+      <c r="D9" s="122" t="s">
         <v>112</v>
       </c>
       <c r="E9" s="42" t="s">
@@ -7073,15 +7101,15 @@
       <c r="H9" s="42" t="s">
         <v>119</v>
       </c>
-      <c r="I9" s="70" t="s">
-        <v>146</v>
+      <c r="I9" s="120" t="s">
+        <v>145</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A10" s="75"/>
-      <c r="B10" s="78"/>
-      <c r="C10" s="80"/>
-      <c r="D10" s="73"/>
+      <c r="A10" s="116"/>
+      <c r="B10" s="119"/>
+      <c r="C10" s="125"/>
+      <c r="D10" s="123"/>
       <c r="E10" s="39" t="s">
         <v>114</v>
       </c>
@@ -7094,147 +7122,147 @@
       <c r="H10" s="39" t="s">
         <v>120</v>
       </c>
-      <c r="I10" s="71"/>
+      <c r="I10" s="121"/>
     </row>
     <row r="11" spans="1:9" ht="69" x14ac:dyDescent="0.3">
-      <c r="A11" s="75"/>
+      <c r="A11" s="116"/>
       <c r="B11" s="52" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="C11" s="34">
         <v>0.4</v>
       </c>
       <c r="D11" s="40" t="s">
+        <v>148</v>
+      </c>
+      <c r="E11" s="41" t="s">
         <v>149</v>
       </c>
-      <c r="E11" s="41" t="s">
+      <c r="F11" s="41" t="s">
         <v>150</v>
       </c>
-      <c r="F11" s="41" t="s">
+      <c r="G11" s="41" t="s">
         <v>151</v>
       </c>
-      <c r="G11" s="41" t="s">
+      <c r="H11" s="41" t="s">
         <v>152</v>
-      </c>
-      <c r="H11" s="41" t="s">
-        <v>153</v>
       </c>
       <c r="I11" s="58">
         <v>7</v>
       </c>
     </row>
     <row r="12" spans="1:9" ht="41.4" x14ac:dyDescent="0.3">
-      <c r="A12" s="75"/>
+      <c r="A12" s="116"/>
       <c r="B12" s="52" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="C12" s="34">
         <v>0.15</v>
       </c>
       <c r="D12" s="40" t="s">
+        <v>154</v>
+      </c>
+      <c r="E12" s="41" t="s">
         <v>155</v>
       </c>
-      <c r="E12" s="41" t="s">
+      <c r="F12" s="41" t="s">
         <v>156</v>
       </c>
-      <c r="F12" s="41" t="s">
+      <c r="G12" s="41" t="s">
         <v>157</v>
       </c>
-      <c r="G12" s="41" t="s">
+      <c r="H12" s="41" t="s">
         <v>158</v>
-      </c>
-      <c r="H12" s="41" t="s">
-        <v>159</v>
       </c>
       <c r="I12" s="58">
         <v>5</v>
       </c>
     </row>
     <row r="13" spans="1:9" ht="55.2" x14ac:dyDescent="0.3">
-      <c r="A13" s="75"/>
+      <c r="A13" s="116"/>
       <c r="B13" s="52" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="C13" s="34">
         <v>0.15</v>
       </c>
       <c r="D13" s="40" t="s">
+        <v>160</v>
+      </c>
+      <c r="E13" s="41" t="s">
         <v>161</v>
       </c>
-      <c r="E13" s="41" t="s">
+      <c r="F13" s="41" t="s">
         <v>162</v>
       </c>
-      <c r="F13" s="41" t="s">
+      <c r="G13" s="41" t="s">
         <v>163</v>
       </c>
-      <c r="G13" s="41" t="s">
+      <c r="H13" s="41" t="s">
         <v>164</v>
-      </c>
-      <c r="H13" s="41" t="s">
-        <v>165</v>
       </c>
       <c r="I13" s="58">
         <v>9</v>
       </c>
     </row>
     <row r="14" spans="1:9" ht="55.2" x14ac:dyDescent="0.3">
-      <c r="A14" s="75"/>
+      <c r="A14" s="116"/>
       <c r="B14" s="52" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="C14" s="34">
         <v>0.1</v>
       </c>
       <c r="D14" s="40" t="s">
+        <v>166</v>
+      </c>
+      <c r="E14" s="41" t="s">
         <v>167</v>
       </c>
-      <c r="E14" s="41" t="s">
+      <c r="F14" s="41" t="s">
         <v>168</v>
       </c>
-      <c r="F14" s="41" t="s">
+      <c r="G14" s="41" t="s">
         <v>169</v>
       </c>
-      <c r="G14" s="41" t="s">
+      <c r="H14" s="41" t="s">
         <v>170</v>
-      </c>
-      <c r="H14" s="41" t="s">
-        <v>171</v>
       </c>
       <c r="I14" s="58">
         <v>7</v>
       </c>
     </row>
     <row r="15" spans="1:9" ht="69.599999999999994" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A15" s="75"/>
+      <c r="A15" s="116"/>
       <c r="B15" s="53" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="C15" s="34">
         <v>0.2</v>
       </c>
       <c r="D15" s="43" t="s">
+        <v>172</v>
+      </c>
+      <c r="E15" s="44" t="s">
         <v>173</v>
       </c>
-      <c r="E15" s="44" t="s">
+      <c r="F15" s="44" t="s">
         <v>174</v>
       </c>
-      <c r="F15" s="44" t="s">
+      <c r="G15" s="44" t="s">
         <v>175</v>
       </c>
-      <c r="G15" s="44" t="s">
+      <c r="H15" s="44" t="s">
         <v>176</v>
-      </c>
-      <c r="H15" s="44" t="s">
-        <v>177</v>
       </c>
       <c r="I15" s="58">
         <v>6</v>
       </c>
     </row>
     <row r="16" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A16" s="76"/>
+      <c r="A16" s="117"/>
       <c r="B16" s="55" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="C16" s="37"/>
       <c r="D16" s="32"/>
@@ -7242,21 +7270,21 @@
       <c r="F16" s="32"/>
       <c r="G16" s="32"/>
       <c r="H16" s="38"/>
-      <c r="I16" s="82">
+      <c r="I16" s="59">
         <f>IF(COUNT(I11:I15)&gt;0,I11*C11+I12*C12+I13*C13+I14*C14+I15*C15,"")</f>
         <v>6.8000000000000007</v>
       </c>
     </row>
     <row r="17" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="18" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A18" s="74" t="s">
-        <v>209</v>
-      </c>
-      <c r="B18" s="77" t="s">
+      <c r="A18" s="115" t="s">
+        <v>289</v>
+      </c>
+      <c r="B18" s="118" t="s">
         <v>111</v>
       </c>
-      <c r="C18" s="79"/>
-      <c r="D18" s="72" t="s">
+      <c r="C18" s="124"/>
+      <c r="D18" s="122" t="s">
         <v>112</v>
       </c>
       <c r="E18" s="42" t="s">
@@ -7271,15 +7299,15 @@
       <c r="H18" s="42" t="s">
         <v>119</v>
       </c>
-      <c r="I18" s="70" t="s">
-        <v>146</v>
+      <c r="I18" s="120" t="s">
+        <v>145</v>
       </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A19" s="75"/>
-      <c r="B19" s="78"/>
-      <c r="C19" s="80"/>
-      <c r="D19" s="73"/>
+      <c r="A19" s="116"/>
+      <c r="B19" s="119"/>
+      <c r="C19" s="125"/>
+      <c r="D19" s="123"/>
       <c r="E19" s="39" t="s">
         <v>114</v>
       </c>
@@ -7292,137 +7320,137 @@
       <c r="H19" s="39" t="s">
         <v>120</v>
       </c>
-      <c r="I19" s="71"/>
+      <c r="I19" s="121"/>
     </row>
     <row r="20" spans="1:9" ht="82.8" x14ac:dyDescent="0.3">
-      <c r="A20" s="75"/>
+      <c r="A20" s="116"/>
       <c r="B20" s="52" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="C20" s="34">
         <v>0.4</v>
       </c>
       <c r="D20" s="40" t="s">
+        <v>178</v>
+      </c>
+      <c r="E20" s="41" t="s">
+        <v>179</v>
+      </c>
+      <c r="F20" s="41" t="s">
         <v>180</v>
       </c>
-      <c r="E20" s="41" t="s">
+      <c r="G20" s="41" t="s">
         <v>181</v>
       </c>
-      <c r="F20" s="41" t="s">
+      <c r="H20" s="41" t="s">
         <v>182</v>
       </c>
-      <c r="G20" s="41" t="s">
+      <c r="I20" s="58"/>
+    </row>
+    <row r="21" spans="1:9" ht="82.8" x14ac:dyDescent="0.3">
+      <c r="A21" s="116"/>
+      <c r="B21" s="52" t="s">
         <v>183</v>
-      </c>
-      <c r="H20" s="41" t="s">
-        <v>184</v>
-      </c>
-      <c r="I20" s="58"/>
-    </row>
-    <row r="21" spans="1:9" ht="82.8" x14ac:dyDescent="0.3">
-      <c r="A21" s="75"/>
-      <c r="B21" s="52" t="s">
-        <v>185</v>
       </c>
       <c r="C21" s="34">
         <v>0.1</v>
       </c>
       <c r="D21" s="40" t="s">
+        <v>184</v>
+      </c>
+      <c r="E21" s="41" t="s">
+        <v>185</v>
+      </c>
+      <c r="F21" s="41" t="s">
         <v>186</v>
       </c>
-      <c r="E21" s="41" t="s">
+      <c r="G21" s="41" t="s">
         <v>187</v>
       </c>
-      <c r="F21" s="41" t="s">
+      <c r="H21" s="41" t="s">
         <v>188</v>
       </c>
-      <c r="G21" s="41" t="s">
+      <c r="I21" s="58"/>
+    </row>
+    <row r="22" spans="1:9" ht="69" x14ac:dyDescent="0.3">
+      <c r="A22" s="116"/>
+      <c r="B22" s="52" t="s">
         <v>189</v>
-      </c>
-      <c r="H21" s="41" t="s">
-        <v>190</v>
-      </c>
-      <c r="I21" s="58"/>
-    </row>
-    <row r="22" spans="1:9" ht="69" x14ac:dyDescent="0.3">
-      <c r="A22" s="75"/>
-      <c r="B22" s="52" t="s">
-        <v>191</v>
       </c>
       <c r="C22" s="34">
         <v>0.1</v>
       </c>
       <c r="D22" s="40" t="s">
+        <v>190</v>
+      </c>
+      <c r="E22" s="41" t="s">
+        <v>191</v>
+      </c>
+      <c r="F22" s="41" t="s">
         <v>192</v>
       </c>
-      <c r="E22" s="41" t="s">
+      <c r="G22" s="41" t="s">
         <v>193</v>
       </c>
-      <c r="F22" s="41" t="s">
+      <c r="H22" s="41" t="s">
         <v>194</v>
       </c>
-      <c r="G22" s="41" t="s">
+      <c r="I22" s="58"/>
+    </row>
+    <row r="23" spans="1:9" ht="69" x14ac:dyDescent="0.3">
+      <c r="A23" s="116"/>
+      <c r="B23" s="52" t="s">
         <v>195</v>
-      </c>
-      <c r="H22" s="41" t="s">
-        <v>196</v>
-      </c>
-      <c r="I22" s="58"/>
-    </row>
-    <row r="23" spans="1:9" ht="69" x14ac:dyDescent="0.3">
-      <c r="A23" s="75"/>
-      <c r="B23" s="52" t="s">
-        <v>197</v>
       </c>
       <c r="C23" s="34">
         <v>0.2</v>
       </c>
       <c r="D23" s="40" t="s">
+        <v>196</v>
+      </c>
+      <c r="E23" s="41" t="s">
+        <v>197</v>
+      </c>
+      <c r="F23" s="41" t="s">
         <v>198</v>
       </c>
-      <c r="E23" s="41" t="s">
+      <c r="G23" s="41" t="s">
         <v>199</v>
       </c>
-      <c r="F23" s="41" t="s">
+      <c r="H23" s="41" t="s">
         <v>200</v>
       </c>
-      <c r="G23" s="41" t="s">
+      <c r="I23" s="58"/>
+    </row>
+    <row r="24" spans="1:9" ht="55.8" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A24" s="116"/>
+      <c r="B24" s="53" t="s">
         <v>201</v>
-      </c>
-      <c r="H23" s="41" t="s">
-        <v>202</v>
-      </c>
-      <c r="I23" s="58"/>
-    </row>
-    <row r="24" spans="1:9" ht="55.8" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A24" s="75"/>
-      <c r="B24" s="53" t="s">
-        <v>203</v>
       </c>
       <c r="C24" s="34">
         <v>0.2</v>
       </c>
       <c r="D24" s="43" t="s">
+        <v>202</v>
+      </c>
+      <c r="E24" s="44" t="s">
+        <v>203</v>
+      </c>
+      <c r="F24" s="44" t="s">
         <v>204</v>
       </c>
-      <c r="E24" s="44" t="s">
+      <c r="G24" s="44" t="s">
         <v>205</v>
       </c>
-      <c r="F24" s="44" t="s">
+      <c r="H24" s="44" t="s">
         <v>206</v>
       </c>
-      <c r="G24" s="44" t="s">
-        <v>207</v>
-      </c>
-      <c r="H24" s="44" t="s">
-        <v>208</v>
-      </c>
       <c r="I24" s="58"/>
     </row>
     <row r="25" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A25" s="76"/>
+      <c r="A25" s="117"/>
       <c r="B25" s="55" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="C25" s="37"/>
       <c r="D25" s="32"/>
@@ -7430,21 +7458,21 @@
       <c r="F25" s="32"/>
       <c r="G25" s="32"/>
       <c r="H25" s="38"/>
-      <c r="I25" s="82" t="str">
+      <c r="I25" s="59" t="str">
         <f>IF(COUNT(I20:I24)&gt;0,I20*C20+I21*C21+I22*C22+I23*C23+I24*C24,"")</f>
         <v/>
       </c>
     </row>
     <row r="26" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="27" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A27" s="74" t="s">
-        <v>240</v>
-      </c>
-      <c r="B27" s="77" t="s">
+      <c r="A27" s="115" t="s">
+        <v>290</v>
+      </c>
+      <c r="B27" s="118" t="s">
         <v>111</v>
       </c>
-      <c r="C27" s="72"/>
-      <c r="D27" s="72" t="s">
+      <c r="C27" s="122"/>
+      <c r="D27" s="122" t="s">
         <v>112</v>
       </c>
       <c r="E27" s="42" t="s">
@@ -7459,15 +7487,15 @@
       <c r="H27" s="42" t="s">
         <v>119</v>
       </c>
-      <c r="I27" s="70" t="s">
-        <v>146</v>
+      <c r="I27" s="120" t="s">
+        <v>145</v>
       </c>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A28" s="75"/>
-      <c r="B28" s="78"/>
-      <c r="C28" s="73"/>
-      <c r="D28" s="73"/>
+      <c r="A28" s="116"/>
+      <c r="B28" s="119"/>
+      <c r="C28" s="123"/>
+      <c r="D28" s="123"/>
       <c r="E28" s="39" t="s">
         <v>114</v>
       </c>
@@ -7480,135 +7508,135 @@
       <c r="H28" s="39" t="s">
         <v>120</v>
       </c>
-      <c r="I28" s="71"/>
+      <c r="I28" s="121"/>
     </row>
     <row r="29" spans="1:9" ht="69" x14ac:dyDescent="0.3">
-      <c r="A29" s="75"/>
+      <c r="A29" s="116"/>
       <c r="B29" s="52" t="s">
-        <v>210</v>
+        <v>207</v>
       </c>
       <c r="C29" s="34">
         <v>0.4</v>
       </c>
       <c r="D29" s="40" t="s">
+        <v>208</v>
+      </c>
+      <c r="E29" s="41" t="s">
+        <v>209</v>
+      </c>
+      <c r="F29" s="41" t="s">
+        <v>210</v>
+      </c>
+      <c r="G29" s="41" t="s">
         <v>211</v>
       </c>
-      <c r="E29" s="41" t="s">
+      <c r="H29" s="41" t="s">
         <v>212</v>
       </c>
-      <c r="F29" s="41" t="s">
+      <c r="I29" s="58"/>
+    </row>
+    <row r="30" spans="1:9" ht="69" x14ac:dyDescent="0.3">
+      <c r="A30" s="116"/>
+      <c r="B30" s="52" t="s">
         <v>213</v>
-      </c>
-      <c r="G29" s="41" t="s">
-        <v>214</v>
-      </c>
-      <c r="H29" s="41" t="s">
-        <v>215</v>
-      </c>
-      <c r="I29" s="58"/>
-    </row>
-    <row r="30" spans="1:9" ht="69" x14ac:dyDescent="0.3">
-      <c r="A30" s="75"/>
-      <c r="B30" s="52" t="s">
-        <v>216</v>
       </c>
       <c r="C30" s="34">
         <v>0.1</v>
       </c>
       <c r="D30" s="40" t="s">
+        <v>214</v>
+      </c>
+      <c r="E30" s="41" t="s">
+        <v>215</v>
+      </c>
+      <c r="F30" s="41" t="s">
+        <v>216</v>
+      </c>
+      <c r="G30" s="41" t="s">
         <v>217</v>
       </c>
-      <c r="E30" s="41" t="s">
+      <c r="H30" s="41" t="s">
         <v>218</v>
       </c>
-      <c r="F30" s="41" t="s">
+      <c r="I30" s="58"/>
+    </row>
+    <row r="31" spans="1:9" ht="96.6" x14ac:dyDescent="0.3">
+      <c r="A31" s="116"/>
+      <c r="B31" s="52" t="s">
         <v>219</v>
-      </c>
-      <c r="G30" s="41" t="s">
-        <v>220</v>
-      </c>
-      <c r="H30" s="41" t="s">
-        <v>221</v>
-      </c>
-      <c r="I30" s="58"/>
-    </row>
-    <row r="31" spans="1:9" ht="96.6" x14ac:dyDescent="0.3">
-      <c r="A31" s="75"/>
-      <c r="B31" s="52" t="s">
-        <v>222</v>
       </c>
       <c r="C31" s="34">
         <v>0.3</v>
       </c>
       <c r="D31" s="40" t="s">
+        <v>220</v>
+      </c>
+      <c r="E31" s="40" t="s">
+        <v>221</v>
+      </c>
+      <c r="F31" s="41" t="s">
+        <v>222</v>
+      </c>
+      <c r="G31" s="41" t="s">
         <v>223</v>
       </c>
-      <c r="E31" s="40" t="s">
+      <c r="H31" s="41" t="s">
         <v>224</v>
       </c>
-      <c r="F31" s="41" t="s">
+      <c r="I31" s="58"/>
+    </row>
+    <row r="32" spans="1:9" ht="55.2" x14ac:dyDescent="0.3">
+      <c r="A32" s="116"/>
+      <c r="B32" s="52" t="s">
         <v>225</v>
-      </c>
-      <c r="G31" s="41" t="s">
-        <v>226</v>
-      </c>
-      <c r="H31" s="41" t="s">
-        <v>227</v>
-      </c>
-      <c r="I31" s="58"/>
-    </row>
-    <row r="32" spans="1:9" ht="55.2" x14ac:dyDescent="0.3">
-      <c r="A32" s="75"/>
-      <c r="B32" s="52" t="s">
-        <v>228</v>
       </c>
       <c r="C32" s="34">
         <v>0.1</v>
       </c>
       <c r="D32" s="40" t="s">
+        <v>226</v>
+      </c>
+      <c r="E32" s="41" t="s">
+        <v>227</v>
+      </c>
+      <c r="F32" s="41" t="s">
+        <v>228</v>
+      </c>
+      <c r="G32" s="41" t="s">
         <v>229</v>
       </c>
-      <c r="E32" s="41" t="s">
+      <c r="H32" s="41" t="s">
         <v>230</v>
       </c>
-      <c r="F32" s="41" t="s">
+      <c r="I32" s="58"/>
+    </row>
+    <row r="33" spans="1:9" ht="41.4" x14ac:dyDescent="0.3">
+      <c r="A33" s="116"/>
+      <c r="B33" s="52" t="s">
         <v>231</v>
-      </c>
-      <c r="G32" s="41" t="s">
-        <v>232</v>
-      </c>
-      <c r="H32" s="41" t="s">
-        <v>233</v>
-      </c>
-      <c r="I32" s="58"/>
-    </row>
-    <row r="33" spans="1:9" ht="41.4" x14ac:dyDescent="0.3">
-      <c r="A33" s="75"/>
-      <c r="B33" s="52" t="s">
-        <v>234</v>
       </c>
       <c r="C33" s="34">
         <v>0.1</v>
       </c>
       <c r="D33" s="40" t="s">
+        <v>232</v>
+      </c>
+      <c r="E33" s="41" t="s">
+        <v>233</v>
+      </c>
+      <c r="F33" s="41" t="s">
+        <v>234</v>
+      </c>
+      <c r="G33" s="41" t="s">
         <v>235</v>
       </c>
-      <c r="E33" s="41" t="s">
+      <c r="H33" s="41" t="s">
         <v>236</v>
       </c>
-      <c r="F33" s="41" t="s">
-        <v>237</v>
-      </c>
-      <c r="G33" s="41" t="s">
-        <v>238</v>
-      </c>
-      <c r="H33" s="41" t="s">
-        <v>239</v>
-      </c>
       <c r="I33" s="58"/>
     </row>
     <row r="34" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A34" s="76"/>
+      <c r="A34" s="117"/>
       <c r="B34" s="54"/>
       <c r="C34" s="45"/>
       <c r="D34" s="45"/>
@@ -7616,21 +7644,21 @@
       <c r="F34" s="45"/>
       <c r="G34" s="45"/>
       <c r="H34" s="45"/>
-      <c r="I34" s="82" t="str">
+      <c r="I34" s="59" t="str">
         <f>IF(COUNT(I29:I33)&gt;0,I29*C29+I30*C30+I31*C31+I32*C32+I33*C33,"")</f>
         <v/>
       </c>
     </row>
     <row r="35" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="36" spans="1:9" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A36" s="74" t="s">
-        <v>267</v>
-      </c>
-      <c r="B36" s="77" t="s">
+      <c r="A36" s="115" t="s">
+        <v>291</v>
+      </c>
+      <c r="B36" s="118" t="s">
         <v>111</v>
       </c>
-      <c r="C36" s="72"/>
-      <c r="D36" s="72" t="s">
+      <c r="C36" s="122"/>
+      <c r="D36" s="122" t="s">
         <v>112</v>
       </c>
       <c r="E36" s="51" t="s">
@@ -7645,15 +7673,15 @@
       <c r="H36" s="42" t="s">
         <v>119</v>
       </c>
-      <c r="I36" s="70" t="s">
-        <v>146</v>
+      <c r="I36" s="120" t="s">
+        <v>145</v>
       </c>
     </row>
     <row r="37" spans="1:9" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A37" s="75"/>
-      <c r="B37" s="78"/>
-      <c r="C37" s="73"/>
-      <c r="D37" s="73"/>
+      <c r="A37" s="116"/>
+      <c r="B37" s="119"/>
+      <c r="C37" s="123"/>
+      <c r="D37" s="123"/>
       <c r="E37" s="49" t="s">
         <v>114</v>
       </c>
@@ -7666,135 +7694,135 @@
       <c r="H37" s="39" t="s">
         <v>120</v>
       </c>
-      <c r="I37" s="71"/>
+      <c r="I37" s="121"/>
     </row>
     <row r="38" spans="1:9" ht="69" x14ac:dyDescent="0.3">
-      <c r="A38" s="75"/>
+      <c r="A38" s="116"/>
       <c r="B38" s="52" t="s">
-        <v>210</v>
+        <v>207</v>
       </c>
       <c r="C38" s="34">
         <v>0.4</v>
       </c>
       <c r="D38" s="40" t="s">
-        <v>241</v>
+        <v>237</v>
       </c>
       <c r="E38" s="41" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="F38" s="41" t="s">
-        <v>213</v>
+        <v>210</v>
       </c>
       <c r="G38" s="41" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="H38" s="41" t="s">
-        <v>242</v>
+        <v>238</v>
       </c>
       <c r="I38" s="58"/>
     </row>
     <row r="39" spans="1:9" ht="55.2" x14ac:dyDescent="0.3">
-      <c r="A39" s="75"/>
+      <c r="A39" s="116"/>
       <c r="B39" s="52" t="s">
-        <v>243</v>
+        <v>239</v>
       </c>
       <c r="C39" s="34">
         <v>0.1</v>
       </c>
       <c r="D39" s="40" t="s">
+        <v>240</v>
+      </c>
+      <c r="E39" s="41" t="s">
+        <v>241</v>
+      </c>
+      <c r="F39" s="41" t="s">
+        <v>242</v>
+      </c>
+      <c r="G39" s="41" t="s">
+        <v>243</v>
+      </c>
+      <c r="H39" s="41" t="s">
         <v>244</v>
       </c>
-      <c r="E39" s="41" t="s">
+      <c r="I39" s="58"/>
+    </row>
+    <row r="40" spans="1:9" ht="55.2" x14ac:dyDescent="0.3">
+      <c r="A40" s="116"/>
+      <c r="B40" s="52" t="s">
         <v>245</v>
-      </c>
-      <c r="F39" s="41" t="s">
-        <v>246</v>
-      </c>
-      <c r="G39" s="41" t="s">
-        <v>247</v>
-      </c>
-      <c r="H39" s="41" t="s">
-        <v>248</v>
-      </c>
-      <c r="I39" s="58"/>
-    </row>
-    <row r="40" spans="1:9" ht="55.2" x14ac:dyDescent="0.3">
-      <c r="A40" s="75"/>
-      <c r="B40" s="52" t="s">
-        <v>249</v>
       </c>
       <c r="C40" s="34">
         <v>0.2</v>
       </c>
       <c r="D40" s="40" t="s">
+        <v>246</v>
+      </c>
+      <c r="E40" s="41" t="s">
+        <v>247</v>
+      </c>
+      <c r="F40" s="41" t="s">
+        <v>248</v>
+      </c>
+      <c r="G40" s="41" t="s">
+        <v>249</v>
+      </c>
+      <c r="H40" s="41" t="s">
         <v>250</v>
       </c>
-      <c r="E40" s="41" t="s">
+      <c r="I40" s="58"/>
+    </row>
+    <row r="41" spans="1:9" ht="41.4" x14ac:dyDescent="0.3">
+      <c r="A41" s="116"/>
+      <c r="B41" s="52" t="s">
         <v>251</v>
-      </c>
-      <c r="F40" s="41" t="s">
-        <v>252</v>
-      </c>
-      <c r="G40" s="41" t="s">
-        <v>253</v>
-      </c>
-      <c r="H40" s="41" t="s">
-        <v>254</v>
-      </c>
-      <c r="I40" s="58"/>
-    </row>
-    <row r="41" spans="1:9" ht="41.4" x14ac:dyDescent="0.3">
-      <c r="A41" s="75"/>
-      <c r="B41" s="52" t="s">
-        <v>255</v>
       </c>
       <c r="C41" s="34">
         <v>0.1</v>
       </c>
       <c r="D41" s="40" t="s">
+        <v>252</v>
+      </c>
+      <c r="E41" s="41" t="s">
+        <v>253</v>
+      </c>
+      <c r="F41" s="41" t="s">
+        <v>254</v>
+      </c>
+      <c r="G41" s="41" t="s">
+        <v>255</v>
+      </c>
+      <c r="H41" s="41" t="s">
         <v>256</v>
       </c>
-      <c r="E41" s="41" t="s">
+      <c r="I41" s="58"/>
+    </row>
+    <row r="42" spans="1:9" ht="55.8" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A42" s="116"/>
+      <c r="B42" s="53" t="s">
         <v>257</v>
-      </c>
-      <c r="F41" s="41" t="s">
-        <v>258</v>
-      </c>
-      <c r="G41" s="41" t="s">
-        <v>259</v>
-      </c>
-      <c r="H41" s="41" t="s">
-        <v>260</v>
-      </c>
-      <c r="I41" s="58"/>
-    </row>
-    <row r="42" spans="1:9" ht="55.8" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A42" s="75"/>
-      <c r="B42" s="53" t="s">
-        <v>261</v>
       </c>
       <c r="C42" s="46">
         <v>0.2</v>
       </c>
       <c r="D42" s="43" t="s">
+        <v>258</v>
+      </c>
+      <c r="E42" s="44" t="s">
+        <v>259</v>
+      </c>
+      <c r="F42" s="44" t="s">
+        <v>260</v>
+      </c>
+      <c r="G42" s="44" t="s">
+        <v>261</v>
+      </c>
+      <c r="H42" s="44" t="s">
         <v>262</v>
       </c>
-      <c r="E42" s="44" t="s">
-        <v>263</v>
-      </c>
-      <c r="F42" s="44" t="s">
-        <v>264</v>
-      </c>
-      <c r="G42" s="44" t="s">
-        <v>265</v>
-      </c>
-      <c r="H42" s="44" t="s">
-        <v>266</v>
-      </c>
       <c r="I42" s="58"/>
     </row>
     <row r="43" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A43" s="76"/>
+      <c r="A43" s="117"/>
       <c r="B43" s="33"/>
       <c r="C43" s="50"/>
       <c r="D43" s="50"/>
@@ -7802,13 +7830,25 @@
       <c r="F43" s="50"/>
       <c r="G43" s="50"/>
       <c r="H43" s="50"/>
-      <c r="I43" s="82" t="str">
+      <c r="I43" s="59" t="str">
         <f>IF(COUNT(I38:I42)&gt;0,I38*C38+I39*C39+I40*C40+I41*C41+I42*C42,"")</f>
         <v/>
       </c>
     </row>
   </sheetData>
   <mergeCells count="25">
+    <mergeCell ref="I36:I37"/>
+    <mergeCell ref="D36:D37"/>
+    <mergeCell ref="I27:I28"/>
+    <mergeCell ref="A27:A34"/>
+    <mergeCell ref="B36:B37"/>
+    <mergeCell ref="C36:C37"/>
+    <mergeCell ref="A36:A43"/>
+    <mergeCell ref="B27:B28"/>
+    <mergeCell ref="D27:D28"/>
+    <mergeCell ref="D18:D19"/>
+    <mergeCell ref="C27:C28"/>
+    <mergeCell ref="I9:I10"/>
     <mergeCell ref="A9:A16"/>
     <mergeCell ref="B18:B19"/>
     <mergeCell ref="A18:A25"/>
@@ -7822,24 +7862,32 @@
     <mergeCell ref="I18:I19"/>
     <mergeCell ref="C9:C10"/>
     <mergeCell ref="C18:C19"/>
-    <mergeCell ref="B27:B28"/>
-    <mergeCell ref="D27:D28"/>
-    <mergeCell ref="D18:D19"/>
-    <mergeCell ref="C27:C28"/>
-    <mergeCell ref="I9:I10"/>
-    <mergeCell ref="I36:I37"/>
-    <mergeCell ref="D36:D37"/>
-    <mergeCell ref="I27:I28"/>
-    <mergeCell ref="A27:A34"/>
-    <mergeCell ref="B36:B37"/>
-    <mergeCell ref="C36:C37"/>
-    <mergeCell ref="A36:A43"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="ed9a2fb8-b6b8-49e0-9782-a1be223650a2">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="bcf2c21e-7c8c-4aa1-a238-b3a814444400" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x010100E784CF8FC968FA419D7090138A1C5306" ma:contentTypeVersion="11" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="39eb63ef951cee5fc2d9dfe9464e3a65">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="ed9a2fb8-b6b8-49e0-9782-a1be223650a2" xmlns:ns3="bcf2c21e-7c8c-4aa1-a238-b3a814444400" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="0c68340d71e68bd9d23afd1fda0793da" ns2:_="" ns3:_="">
     <xsd:import namespace="ed9a2fb8-b6b8-49e0-9782-a1be223650a2"/>
@@ -8034,41 +8082,10 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="ed9a2fb8-b6b8-49e0-9782-a1be223650a2">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="bcf2c21e-7c8c-4aa1-a238-b3a814444400" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2B717C7F-1EC7-4AD7-98AC-1B0BAECCBAD4}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{90A2FB82-F486-424F-AB4A-CA9A356DA4CC}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="ed9a2fb8-b6b8-49e0-9782-a1be223650a2"/>
-    <ds:schemaRef ds:uri="bcf2c21e-7c8c-4aa1-a238-b3a814444400"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -8091,9 +8108,20 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{90A2FB82-F486-424F-AB4A-CA9A356DA4CC}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2B717C7F-1EC7-4AD7-98AC-1B0BAECCBAD4}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="ed9a2fb8-b6b8-49e0-9782-a1be223650a2"/>
+    <ds:schemaRef ds:uri="bcf2c21e-7c8c-4aa1-a238-b3a814444400"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>